<commit_message>
Share latest step6 output for review
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -166,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -631,12 +631,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="226">
+  <cellXfs count="227">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -1216,12 +1222,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1247,6 +1253,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1607,12 +1616,12 @@
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
     <col width="12.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="39" max="39"/>
-    <col width="32" customWidth="1" min="40" max="40"/>
-    <col width="12" customWidth="1" min="41" max="41"/>
-    <col width="32" customWidth="1" min="42" max="42"/>
-    <col width="38" customWidth="1" min="43" max="43"/>
-    <col width="55" customWidth="1" min="44" max="44"/>
+    <col width="8" customWidth="1" min="39" max="39"/>
+    <col width="45" customWidth="1" min="40" max="40"/>
+    <col width="8" customWidth="1" min="41" max="41"/>
+    <col width="40" customWidth="1" min="42" max="42"/>
+    <col width="45" customWidth="1" min="43" max="43"/>
+    <col width="60" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2048,6 +2057,11 @@
           <t>Suggestion</t>
         </is>
       </c>
+      <c r="AN13" s="205" t="n"/>
+      <c r="AO13" s="205" t="n"/>
+      <c r="AP13" s="205" t="n"/>
+      <c r="AQ13" s="205" t="n"/>
+      <c r="AR13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2088,6 +2102,12 @@
       <c r="AJ14" s="195" t="n"/>
       <c r="AK14" s="195" t="n"/>
       <c r="AL14" s="199" t="n"/>
+      <c r="AM14" s="205" t="n"/>
+      <c r="AN14" s="205" t="n"/>
+      <c r="AO14" s="205" t="n"/>
+      <c r="AP14" s="205" t="n"/>
+      <c r="AQ14" s="205" t="n"/>
+      <c r="AR14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2315,6 +2335,12 @@
       <c r="AJ16" s="212" t="n"/>
       <c r="AK16" s="212" t="n"/>
       <c r="AL16" s="213" t="n"/>
+      <c r="AM16" s="208" t="n"/>
+      <c r="AN16" s="208" t="n"/>
+      <c r="AO16" s="208" t="n"/>
+      <c r="AP16" s="208" t="n"/>
+      <c r="AQ16" s="208" t="n"/>
+      <c r="AR16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2355,6 +2381,12 @@
       <c r="AJ17" s="215" t="n"/>
       <c r="AK17" s="215" t="n"/>
       <c r="AL17" s="216" t="n"/>
+      <c r="AM17" s="208" t="n"/>
+      <c r="AN17" s="208" t="n"/>
+      <c r="AO17" s="208" t="n"/>
+      <c r="AP17" s="208" t="n"/>
+      <c r="AQ17" s="208" t="n"/>
+      <c r="AR17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2476,22 +2508,27 @@
       <c r="AJ18" s="45" t="n"/>
       <c r="AK18" s="45" t="n"/>
       <c r="AL18" s="35" t="n"/>
-      <c r="AM18" s="169" t="n">
+      <c r="AM18" s="223" t="n">
         <v>8</v>
       </c>
-      <c r="AN18" s="169" t="inlineStr">
-        <is>
-          <t>The End User effects list functional outcomes (no light or dim light) without any explicit safety or regulatory language; given the merged "scratch/damage" mode, the DAMAGE sub-mode can directly cause either total loss or degradation of the headlamp’s primary function, so the worst-case applicable definition is loss of primary function (8).</t>
-        </is>
-      </c>
-      <c r="AQ18" s="169" t="inlineStr">
-        <is>
-          <t>Add a mandatory barcode scan at the sequencing trolley that interlocks the station and blocks tool enable if the scanned headlamp PN/variant does not match the vehicle build sheet, preventing wrong-part selection/mix-up.</t>
-        </is>
-      </c>
-      <c r="AR18" s="169" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Scratch on head lamp; 2. Damage on head lamp. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it reads like the cause for installing the wrong headlamp variant rather than for scratching/damaging the part. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+      <c r="AN18" s="223" t="inlineStr">
+        <is>
+          <t>Among the listed End User effects, the merged mode "scratch/damage" can directly cause either a total loss (does not turn ON) or a degradation (dim light) of the headlamp’s primary function; per the worst-case rule for merged modes, the total loss case maps to Severity 8.</t>
+        </is>
+      </c>
+      <c r="AP18" s="223" t="inlineStr">
+        <is>
+          <t>Install an automated vision inspection at the install station (diffuse lighting dome) to detect lens scratches/cracks and obvious physical damage on the headlamp before torqueing and release.</t>
+        </is>
+      </c>
+      <c r="AQ18" s="223" t="inlineStr">
+        <is>
+          <t>Add a pick-to-light with barcode interlock on the sequencing trolley that only unlocks and illuminates the correct LH/RH headlamp variant slot for the current build, preventing wrong-part picks and mix-ups.</t>
+        </is>
+      </c>
+      <c r="AR18" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Cause/Mode mismatch: The stated cause (wrong part selection/mix-up) does not physically produce a scratch/damage; it aligns with a separate wrong-variant installation failure mode rather than cosmetic/physical damage. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2541,6 +2578,11 @@
       <c r="AJ19" s="45" t="n"/>
       <c r="AK19" s="45" t="n"/>
       <c r="AL19" s="35" t="n"/>
+      <c r="AM19" s="223" t="n"/>
+      <c r="AN19" s="223" t="n"/>
+      <c r="AP19" s="223" t="n"/>
+      <c r="AQ19" s="223" t="n"/>
+      <c r="AR19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2583,22 +2625,27 @@
       <c r="AJ20" s="45" t="n"/>
       <c r="AK20" s="45" t="n"/>
       <c r="AL20" s="35" t="n"/>
-      <c r="AM20" s="169" t="n">
+      <c r="AM20" s="223" t="n">
         <v>8</v>
       </c>
-      <c r="AN20" s="169" t="inlineStr">
-        <is>
-          <t>The End User effects list either a total loss of the headlamp function ('does not turn ON') or a degraded primary function ('dim light'), both directly plausible from wrong-part selection/mix-up; no safety or regulatory wording is stated. Per the table, these correspond to S=8 or S=7 respectively, with the row-level score set to the higher (8) due to merged/ambiguous mode effects.</t>
-        </is>
-      </c>
-      <c r="AQ20" s="169" t="inlineStr">
-        <is>
-          <t>Add a scan-and-verify lockout at the pick/scan step so the headlamp barcode must match the vehicle’s model code and the line prevents installation if a wrong part is scanned.</t>
-        </is>
-      </c>
-      <c r="AR20" s="169" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+      <c r="AN20" s="223" t="inlineStr">
+        <is>
+          <t>The End User effects explicitly include both total loss of the headlamp’s function (does not turn ON) and a degraded state (dim light); with no safety or regulatory text given, the AIAG-VDA table maps these to 8 and 7, respectively, and the worst-case direct outcome is 8.</t>
+        </is>
+      </c>
+      <c r="AP20" s="223" t="inlineStr">
+        <is>
+          <t>Introduce an automated functional illumination test after installation that powers the headlamp and uses a current sensor plus a lux/vision sensor to verify both ON-state and minimum intensity before release.</t>
+        </is>
+      </c>
+      <c r="AQ20" s="223" t="inlineStr">
+        <is>
+          <t>Add a barcode/RFID scan interlock tied to the vehicle build record that prevents tool enable/line advance if the scanned headlamp PN does not match the model, eliminating wrong-part picks from the sequencing trolley.</t>
+        </is>
+      </c>
+      <c r="AR20" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of headlamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2646,6 +2693,11 @@
       <c r="AJ21" s="45" t="n"/>
       <c r="AK21" s="45" t="n"/>
       <c r="AL21" s="35" t="n"/>
+      <c r="AM21" s="223" t="n"/>
+      <c r="AN21" s="223" t="n"/>
+      <c r="AP21" s="223" t="n"/>
+      <c r="AQ21" s="223" t="n"/>
+      <c r="AR21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2663,7 +2715,7 @@
       <c r="J22" s="207" t="n"/>
       <c r="K22" s="211" t="n"/>
       <c r="L22" s="210" t="n"/>
-      <c r="M22" s="223" t="inlineStr">
+      <c r="M22" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. Wiring harness partially connected (loose fitment)
@@ -2704,22 +2756,27 @@
       <c r="AJ22" s="45" t="n"/>
       <c r="AK22" s="45" t="n"/>
       <c r="AL22" s="35" t="n"/>
-      <c r="AM22" s="169" t="n">
+      <c r="AM22" s="223" t="n">
         <v>10</v>
       </c>
-      <c r="AN22" s="169" t="inlineStr">
-        <is>
-          <t>The End User effect list explicitly states 'Increased risk of accident', which is a plausible consequence of the headlamp not turning on or reduced visibility caused by improper/poor connector locking. Per the table, this affects safe operation of the vehicle, so Severity is 10.</t>
-        </is>
-      </c>
-      <c r="AQ22" s="169" t="inlineStr">
-        <is>
-          <t>Add a poka‑yoke for the headlamp connectors: a latch‑engagement sensor or pull‑back test with line interlock that prevents process completion if the connector is not fully seated and locked.</t>
-        </is>
-      </c>
-      <c r="AR22" s="169" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+      <c r="AN22" s="223" t="inlineStr">
+        <is>
+          <t>Improper/poor locking of the headlamp connectors (or forgetting the socket connection) can leave the headlamp unpowered, reducing road visibility; the End User effect list explicitly states 'Increased risk of accident', which maps to the table’s safety criterion.</t>
+        </is>
+      </c>
+      <c r="AP22" s="223" t="inlineStr">
+        <is>
+          <t>Implement an automated end-of-station functional test that powers the headlamp (low/high as applicable) and verifies current draw/illumination to detect unconnected or poorly locked connectors.</t>
+        </is>
+      </c>
+      <c r="AQ22" s="223" t="inlineStr">
+        <is>
+          <t>Add a poka‑yoke connector seating fixture with PLC interlock that drives each headlamp connector to full depth and verifies latch engagement (force–displacement/latch switch) before allowing the station to proceed.</t>
+        </is>
+      </c>
+      <c r="AR22" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Improper locking; 2. Poor locking. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -2787,6 +2844,11 @@
       <c r="AJ23" s="12" t="n"/>
       <c r="AK23" s="12" t="n"/>
       <c r="AL23" s="10" t="n"/>
+      <c r="AM23" s="223" t="n"/>
+      <c r="AN23" s="223" t="n"/>
+      <c r="AP23" s="223" t="n"/>
+      <c r="AQ23" s="223" t="n"/>
+      <c r="AR23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -2835,20 +2897,25 @@
       <c r="AJ24" s="12" t="n"/>
       <c r="AK24" s="12" t="n"/>
       <c r="AL24" s="10" t="n"/>
-      <c r="AM24" s="169" t="n">
+      <c r="AM24" s="223" t="n">
         <v>10</v>
       </c>
-      <c r="AN24" s="169" t="inlineStr">
-        <is>
-          <t>The End User effect explicitly states 'Increased risk of accident,' which is a direct and plausible consequence of a headlamp installed without required prefit bolts causing misalignment or compromised illumination. Per the Severity table, this affects safe operation of the vehicle, warranting a 10.</t>
-        </is>
-      </c>
-      <c r="AQ24" s="169" t="inlineStr">
-        <is>
-          <t>Install a DC torque tool with bolt-count and torque OK interlock that prevents station completion unless all headlamp bolts are started and torqued to 6 Nm per the SOS.</t>
-        </is>
-      </c>
-      <c r="AR24" s="169" t="inlineStr">
+      <c r="AN24" s="223" t="inlineStr">
+        <is>
+          <t>The End User effects explicitly include "Increased risk of accident," which is a plausible consequence of an unbolted headlamp causing incorrect beam alignment or non-function and reduced road visibility; this matches the table’s safety/health risk criterion.</t>
+        </is>
+      </c>
+      <c r="AP24" s="223" t="inlineStr">
+        <is>
+          <t>Add a vision camera or bolt-presence sensor check that verifies all headlamp bolt heads are present and seated before line release, with NOK stop if any are missing.</t>
+        </is>
+      </c>
+      <c r="AQ24" s="223" t="inlineStr">
+        <is>
+          <t>Install a torque-controlled, bolt-counting electric driver interlocked to the station PLC so the job cannot be completed unless all headlamp bolts achieve 6 Nm OK.</t>
+        </is>
+      </c>
+      <c r="AR24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2902,6 +2969,11 @@
       <c r="AJ25" s="12" t="n"/>
       <c r="AK25" s="12" t="n"/>
       <c r="AL25" s="10" t="n"/>
+      <c r="AM25" s="223" t="n"/>
+      <c r="AN25" s="223" t="n"/>
+      <c r="AP25" s="223" t="n"/>
+      <c r="AQ25" s="223" t="n"/>
+      <c r="AR25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -2919,7 +2991,7 @@
       <c r="J26" s="207" t="n"/>
       <c r="K26" s="211" t="n"/>
       <c r="L26" s="210" t="n"/>
-      <c r="M26" s="223" t="inlineStr">
+      <c r="M26" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
@@ -2962,22 +3034,27 @@
       <c r="AJ26" s="12" t="n"/>
       <c r="AK26" s="12" t="n"/>
       <c r="AL26" s="10" t="n"/>
-      <c r="AM26" s="169" t="n">
+      <c r="AM26" s="223" t="n">
         <v>4</v>
       </c>
-      <c r="AN26" s="169" t="inlineStr">
-        <is>
-          <t>Among the listed End User effects, the only direct outcome of 'failed to fit screws/not maintained gap' is 'rattling or vibration noise during driving', which falls under very objectionable sound/vibration. The more severe-sounding effects (lens crack, bulb burnout, water ingress) require additional unstated failures and are therefore indirect for this mode/cause.</t>
-        </is>
-      </c>
-      <c r="AQ26" s="169" t="inlineStr">
-        <is>
-          <t>Add an in-station fixture with hard locators and an interlocked gap/fastener verification (camera or go/no-go gauge plus screw-counting torque tool) that blocks OK-to-ship unless uniform gaps are met and all screws are installed/torqued.</t>
-        </is>
-      </c>
-      <c r="AR26" s="169" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap. Cause/Mode mismatch: The stated Cause addresses only non-uniform gaps to the fender; it does not explain the 'failed to fit screws' portion of the Failure Mode.</t>
+      <c r="AN26" s="223" t="inlineStr">
+        <is>
+          <t>The only DIRECT End User effect of the stated fit/fastener condition is rattling/vibration noise while driving, which is an NVH complaint. The list contains no explicit safety or regulatory wording tied directly to this cause, so Severity aligns with 'very objectionable' NVH.</t>
+        </is>
+      </c>
+      <c r="AP26" s="223" t="inlineStr">
+        <is>
+          <t>Install an automated vision check to verify both mounting screws are present and measure the lamp-to-fender gap around the perimeter with pass/fail limits before station release.</t>
+        </is>
+      </c>
+      <c r="AQ26" s="223" t="inlineStr">
+        <is>
+          <t>Add a dedicated headlamp locating fixture with hard datums to the BIW and clamp pads that lock the lamp in the correct position so uniform gap is fixed before tightening the screws.</t>
+        </is>
+      </c>
+      <c r="AR26" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap.</t>
         </is>
       </c>
     </row>
@@ -3035,6 +3112,11 @@
       <c r="AJ27" s="12" t="n"/>
       <c r="AK27" s="12" t="n"/>
       <c r="AL27" s="10" t="n"/>
+      <c r="AM27" s="223" t="n"/>
+      <c r="AN27" s="223" t="n"/>
+      <c r="AP27" s="223" t="n"/>
+      <c r="AQ27" s="223" t="n"/>
+      <c r="AR27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3044,7 +3126,7 @@
       <c r="F28" s="210" t="n"/>
       <c r="G28" s="211" t="n"/>
       <c r="H28" s="210" t="n"/>
-      <c r="I28" s="224" t="inlineStr">
+      <c r="I28" s="225" t="inlineStr">
         <is>
           <t>PROPER TIGHTENING OF JOINT</t>
         </is>
@@ -3096,20 +3178,25 @@
       <c r="AJ28" s="12" t="n"/>
       <c r="AK28" s="12" t="n"/>
       <c r="AL28" s="10" t="n"/>
-      <c r="AM28" s="169" t="n">
+      <c r="AM28" s="223" t="n">
         <v>4</v>
       </c>
-      <c r="AN28" s="169" t="inlineStr">
-        <is>
-          <t>The direct customer-facing outcome of an under-torqued headlamp mount is rattle/vibration noise while driving, which fits the table’s NVH category. This is reasonably treated as very objectionable NVH, aligning with Severity 4.</t>
-        </is>
-      </c>
-      <c r="AQ28" s="169" t="inlineStr">
-        <is>
-          <t>Install a torque-controlled, calibrated electric driver programmed to 6 Nm with OK/NOK lockout to prevent under-torque from operator mistake, wrong tool use, or miscalibration.</t>
-        </is>
-      </c>
-      <c r="AR28" s="169" t="inlineStr">
+      <c r="AN28" s="223" t="inlineStr">
+        <is>
+          <t>The most direct End User outcome of an under-torqued headlamp is rattling/vibration noise while driving. This is an NVH issue that customers would find very objectionable, which matches the table’s definition for severity 4.</t>
+        </is>
+      </c>
+      <c r="AP28" s="223" t="inlineStr">
+        <is>
+          <t>Add in-station torque/angle monitoring with transducer feedback that records OK/NOK per fastener and interlocks the line on NOK so under-torque cannot pass.</t>
+        </is>
+      </c>
+      <c r="AQ28" s="223" t="inlineStr">
+        <is>
+          <t>Install a DC-electric torque tool with program locked to 6 Nm and a PLC interlock that only enables the correct tool/program at this station to prevent operator error and use of the wrong tool.</t>
+        </is>
+      </c>
+      <c r="AR28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3154,28 +3241,34 @@
       <c r="AJ29" s="12" t="n"/>
       <c r="AK29" s="12" t="n"/>
       <c r="AL29" s="10" t="n"/>
-      <c r="AM29" s="169" t="n">
+      <c r="AM29" s="223" t="n">
         <v>4</v>
       </c>
-      <c r="AN29" s="169" t="inlineStr">
-        <is>
-          <t>The direct customer outcomes of this torque error are a cracked/broken lens (over‑torque) or rattling/vibration noise (under‑torque), which are NVH/appearance issues; there is no explicit accident/injury or regulatory noncompliance stated, and loss/degradation of illumination is not directly attributed to this torque error in the listed effects.</t>
-        </is>
-      </c>
-      <c r="AQ29" s="169" t="inlineStr">
-        <is>
-          <t>Install a DC torque tool programmed to 6 Nm with barcode-linked job selection and OK/NOK lockout so the station cannot proceed if the specified torque is not achieved, preventing wrong tool use and calibration drift from producing under/over‑torque.</t>
-        </is>
-      </c>
-      <c r="AR29" s="169" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Under‑torque (torque not achieved); 2. Over‑torque. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+      <c r="AN29" s="223" t="inlineStr">
+        <is>
+          <t>For the merged mode “TORQUE NOT ACHIEVED – OVER TORQUE”, the DIRECT End User outcomes are a cracked/broken lens (over‑torque) and rattling/vibration noise (under‑torque); both are very objectionable appearance/NVH issues and the list does not state an accident/injury, regulatory noncompliance, or an explicit primary‑function loss.</t>
+        </is>
+      </c>
+      <c r="AP29" s="223" t="inlineStr">
+        <is>
+          <t>Add 100% electronic torque/angle monitoring with OK/NOK and trace storage in MES, interlocked to stop the line or require rework if the achieved torque is out of the 6 Nm tolerance window.</t>
+        </is>
+      </c>
+      <c r="AQ29" s="223" t="inlineStr">
+        <is>
+          <t>Implement a torque/angle‑controlled DC tool with job program lock at 6 Nm, interlocked to the station by barcode/RFID so the joint cannot be run with the wrong tool or wrong setting.</t>
+        </is>
+      </c>
+      <c r="AR29" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED; 2. OVER TORQUE. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="152">
+  <mergeCells count="157">
+    <mergeCell ref="AP18:AP19"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
@@ -3222,6 +3315,7 @@
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="AN20:AN21"/>
+    <mergeCell ref="AP20:AP21"/>
     <mergeCell ref="AQ22:AQ23"/>
     <mergeCell ref="AN26:AN27"/>
     <mergeCell ref="A5:C5"/>
@@ -3230,6 +3324,7 @@
     <mergeCell ref="Z18:Z21"/>
     <mergeCell ref="T25:U25"/>
     <mergeCell ref="AN22:AN23"/>
+    <mergeCell ref="AP22:AP23"/>
     <mergeCell ref="P18:Q19"/>
     <mergeCell ref="AQ15:AQ17"/>
     <mergeCell ref="Y23:Y25"/>
@@ -3259,12 +3354,14 @@
     <mergeCell ref="A13:F14"/>
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
+    <mergeCell ref="AP24:AP25"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="P15:Q17"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="AH15:AH17"/>
     <mergeCell ref="AJ15:AJ17"/>
     <mergeCell ref="O27:O29"/>
+    <mergeCell ref="AP26:AP27"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="O18:O21"/>
     <mergeCell ref="M18:N21"/>
@@ -4327,7 +4424,7 @@
       <c r="J22" s="207" t="n"/>
       <c r="K22" s="211" t="n"/>
       <c r="L22" s="210" t="n"/>
-      <c r="M22" s="223" t="inlineStr">
+      <c r="M22" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. Wiring harness partially connected (loose fitment)
@@ -4535,7 +4632,7 @@
       <c r="F26" s="210" t="n"/>
       <c r="G26" s="211" t="n"/>
       <c r="H26" s="210" t="n"/>
-      <c r="I26" s="225" t="inlineStr">
+      <c r="I26" s="226" t="inlineStr">
         <is>
           <t>PROPER TIGHTENING OF JOINT</t>
         </is>
@@ -4543,7 +4640,7 @@
       <c r="J26" s="207" t="n"/>
       <c r="K26" s="211" t="n"/>
       <c r="L26" s="210" t="n"/>
-      <c r="M26" s="223" t="inlineStr">
+      <c r="M26" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
@@ -5996,7 +6093,7 @@
       <c r="F24" s="210" t="n"/>
       <c r="G24" s="211" t="n"/>
       <c r="H24" s="210" t="n"/>
-      <c r="I24" s="225" t="inlineStr">
+      <c r="I24" s="226" t="inlineStr">
         <is>
           <t>PROPER TIGHTENING OF JOINT</t>
         </is>
@@ -6004,7 +6101,7 @@
       <c r="J24" s="207" t="n"/>
       <c r="K24" s="211" t="n"/>
       <c r="L24" s="210" t="n"/>
-      <c r="M24" s="223" t="inlineStr">
+      <c r="M24" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
@@ -7242,7 +7339,7 @@
       <c r="J20" s="136" t="n"/>
       <c r="K20" s="211" t="n"/>
       <c r="L20" s="210" t="n"/>
-      <c r="M20" s="223" t="inlineStr">
+      <c r="M20" s="224" t="inlineStr">
         <is>
           <t>Your Plant:
 1. Cut, torn, pinched, or cracked seal
@@ -7463,7 +7560,7 @@
       <c r="F24" s="210" t="n"/>
       <c r="G24" s="211" t="n"/>
       <c r="H24" s="210" t="n"/>
-      <c r="I24" s="225" t="inlineStr">
+      <c r="I24" s="226" t="inlineStr">
         <is>
           <t>PROPER TIGHTENING OF JOINT</t>
         </is>

</xml_diff>

<commit_message>
Re-run with merged-mode split-scoring active
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -2513,22 +2513,22 @@
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>The End User effects include a DIRECT, plausible total loss of headlamp function ('Headlamp does not turn ON') for the 'damage' sub-mode, which per the table is a loss of a primary vehicle function; no safety/accident or regulatory wording is present.</t>
+          <t>The End User effects include 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation). With a merged mode 'SCRATCH / DAMAGE', the 'damage' sub-mode can directly yield a complete loss of headlamp function, mapping to Severity 8 per the table.</t>
         </is>
       </c>
       <c r="AP18" s="223" t="inlineStr">
         <is>
-          <t>Add an automatic headlamp power-on illumination test with a lux sensor at this station and interlock the process if the lamp fails to turn on or measured intensity is below threshold.</t>
+          <t>Install an in-station camera-based vision inspection to automatically detect and reject headlamp lens/housing scratches or cracks before final tightening.</t>
         </is>
       </c>
       <c r="AQ18" s="223" t="inlineStr">
         <is>
-          <t>Implement a keyed, variant-specific sequencing trolley with dedicated, physically incompatible slots for each headlamp part number so the wrong variant cannot be staged or picked in the first place.</t>
+          <t>Add a pick-to-light bin-door interlock on the headlamp sequencing trolley tied to barcode scan and build manifest so the operator cannot access or select the wrong variant.</t>
         </is>
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Scratch on head lamp; 2. Damage on head lamp. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not inherently produce a scratch/damage; it aligns with a 'wrong headlamp variant installed' mode rather than the cosmetic/physical damage described here. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it aligns with a 'wrong headlamp variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2630,22 +2630,22 @@
       </c>
       <c r="AN20" s="223" t="inlineStr">
         <is>
-          <t>The End User effects include both a total loss of lighting (does not turn ON) and degraded lighting (dim), which map to loss or degradation of a primary vehicle function. With no safety or regulatory wording present, the appropriate band is 7–8; using the worst-case direct effect yields 8.</t>
+          <t>The listed End User effects include both total loss of illumination and dim illumination. These map to loss or degradation of a primary vehicle function (headlighting). Without any explicit safety or regulatory wording, the worst-case direct outcome for the merged mode is "does not turn ON," which corresponds to S=8.</t>
         </is>
       </c>
       <c r="AP20" s="223" t="inlineStr">
         <is>
-          <t>Add an automated post-installation headlamp functional/illumination test using a power-on check with a camera/lux sensor to verify each lamp turns ON and meets a set brightness threshold before release.</t>
+          <t>Introduce an automated headlamp functional test at this station that commands ON and verifies illumination with a camera/lux sensor (or current sensor) before release.</t>
         </is>
       </c>
       <c r="AQ20" s="223" t="inlineStr">
         <is>
-          <t>Add a pick-to-light system with electronically latched, model/LH-RH specific bins on the sequencing trolley tied to the build manifest so only the correct headlamp bin opens, preventing wrong-part removal and mix-ups.</t>
+          <t>Add a VIN-linked pick-to-light/locking-bin system on the sequencing trolley so only the correct LH/RH headlamp bin illuminates and unlocks for the model, preventing wrong-part selection.</t>
         </is>
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of headlamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2761,22 +2761,22 @@
       </c>
       <c r="AN22" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include 'Increased risk of accident,' which is a plausible consequence of an unconnected/poorly locked headlamp connector causing the lamp not to turn on and reducing road visibility. Per the Severity table, this affects safe operation of the vehicle, so Severity is 10.</t>
+          <t>Improper/forgotten connector locking can leave the headlamp inoperative, which reduces road visibility; the End User effects explicitly state 'Increased risk of accident'. This matches the Severity 10 definition affecting safe vehicle operation and road user safety.</t>
         </is>
       </c>
       <c r="AP22" s="223" t="inlineStr">
         <is>
-          <t>Install an automatic in-station functional test that powers the headlamp and verifies current draw/illumination with a light sensor; block the station if either connector is not making electrical contact.</t>
+          <t>Add an automated functional test at this station that powers the headlamp circuits and verifies current/illumination with a sensor, stopping the line if either connector is not making electrical contact.</t>
         </is>
       </c>
       <c r="AQ22" s="223" t="inlineStr">
         <is>
-          <t>Add a poka‑yoke interlock that enables the 6 Nm torque tool (or station OK‑to‑move) only after sensors/continuity checks confirm both headlamp connectors are fully latched.</t>
+          <t>Install a keyed connector insertion fixture with a mechanical interlock that only releases the part for bolt tightening when both headlamp connectors are fully seated and latched to the hard-stop.</t>
         </is>
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2902,17 @@
       </c>
       <c r="AN24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include 'Increased risk of accident,' which is a plausible consequence of a headlamp not bolted in place leading to misalignment/reduced road illumination. Per Table C2-1, an effect that impacts safe operation of the vehicle or road users is Severity 10.</t>
+          <t>The End User effects explicitly state 'Increased risk of accident', which is a safety consequence plausibly resulting from mis-aimed or non-functioning headlamps when bolts are not prefitted. Per the scoring rules, an explicit, causally plausible safety phrase requires Severity = 10.</t>
         </is>
       </c>
       <c r="AP24" s="223" t="inlineStr">
         <is>
-          <t>Install a vision/bolt-presence verification camera at the station that confirms all required headlamp bolts are present (and in the correct locations) with a line interlock to prevent release if any bolt is missing.</t>
+          <t>Add an end-of-station vision check that verifies both headlamp bolts are present and seated (and lamp is flush/aligned), with NOK line stop and image traceability.</t>
         </is>
       </c>
       <c r="AQ24" s="223" t="inlineStr">
         <is>
-          <t>Add a pick-to-light kitting system for the headlamp bolts with count confirmation interlocked to the station so the fastening step cannot begin unless the required number of bolts has been picked per SOS.</t>
+          <t>Install a DC electric fastening system with controller that requires the required number of 6 Nm OK tighten events (bolt count) and locks out completion until achieved, with bolt-present/socket-present sensors on the tool.</t>
         </is>
       </c>
       <c r="AR24" s="223" t="inlineStr">
@@ -3039,22 +3039,22 @@
       </c>
       <c r="AN26" s="223" t="inlineStr">
         <is>
-          <t>The only direct End User effect of the stated fit/fastener failure is 'Rattling or vibration noise during driving', which aligns with a very objectionable NVH condition. No explicit safety or regulatory consequences are stated, and illumination loss/degradation is not directly claimed for this fit-and-gap issue.</t>
+          <t>Among the listed End User effects, the direct outcome of missing/loose screws is rattling or vibration noise during driving, which maps to very objectionable sound/vibration per the table. More severe items like bulb burnout or water ingress require additional unstated failure mechanisms and are not used for the representative severity.</t>
         </is>
       </c>
       <c r="AP26" s="223" t="inlineStr">
         <is>
-          <t>Install a camera-based vision check that measures the headlamp-to-fender gap at defined points and verifies screw presence, with automatic NOK/line-stop if gaps or any screw are out of spec/missing.</t>
+          <t>Install an in-station vision system to automatically measure headlamp-to-fender gap/flushness and verify both mounting screws are present/seated, interlocked to stop the line on fail.</t>
         </is>
       </c>
       <c r="AQ26" s="223" t="inlineStr">
         <is>
-          <t>Add a dedicated locating fixture with hard stops (poka-yoke) that positively seats the headlamp to the BIW to enforce the specified uniform gap before bolts can be accessed and tightened.</t>
+          <t>Add a dedicated alignment/locator fixture with hard stops that sets the headlamp-to-fender gap uniformly and clamps the lamp in position during tightening so the operator cannot torque unless the gap is within spec.</t>
         </is>
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. FAILED TO FIT SCREWS; 2. NOT MAINTAINED GAP. Cause/Mode mismatch: The Cause (operator doesn't maintain uniform gaps) does not explain the 'failed to fit screws' sub-mode; it reads as the cause only for the gap-maintenance issue.</t>
+          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap between headlamp and fender edge. Cause/Mode mismatch: The stated cause addresses only non-uniform gaps, not missing/failed-to-fit screws; it appears to belong to the 'not maintained gap' sub-mode rather than the 'failed to fit screws' sub-mode.</t>
         </is>
       </c>
     </row>
@@ -3183,17 +3183,17 @@
       </c>
       <c r="AN28" s="223" t="inlineStr">
         <is>
-          <t>For an under-torqued headlamp mounting, the direct End User effect listed is "Rattling or vibration noise during driving," which fits the table’s NVH category of very objectionable sound/vibration. Other listed effects (lens crack, water ingress, bulb burnout, eye strain) require additional unstated mechanisms, so they are indirect for this mode/cause.</t>
+          <t>Under‑torque leads to a loose headlamp mounting, which directly produces rattling/vibration noise during driving. This maps to "Very objectionable ... vibration/harshness" in the End User column. No explicit safety or regulatory effects are stated for this failure.</t>
         </is>
       </c>
       <c r="AP28" s="223" t="inlineStr">
         <is>
-          <t>Integrate a transducerized DC torque controller that records torque/angle for each fastener with OK/NOK lockout so the station cannot complete if 6 Nm is not achieved.</t>
+          <t>Add torque/angle monitoring with OK/NOK interlock on the tool so the station cannot release an OK until 6 Nm is achieved, with cycle‑by‑cycle traceable data logging.</t>
         </is>
       </c>
       <c r="AQ28" s="223" t="inlineStr">
         <is>
-          <t>Add an RFID/PLC-interlocked DC tool program and keyed socket so only the correct 6 Nm torque program is enabled at this station, preventing use of the wrong tool and operator under-torque.</t>
+          <t>Implement a controller‑locked DC torque tool preset to 6 Nm with station interlock (tool/spindle ID or RFID) so a wrong tool cannot run and the correct torque program is always applied.</t>
         </is>
       </c>
       <c r="AR28" s="223" t="inlineStr">
@@ -3246,22 +3246,22 @@
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
-          <t>The DIRECT End User effects for this torque error are either a cracked/broken lens (over‑torque) or rattling/vibration noise (under‑torque), both of which are very objectionable NVH/appearance outcomes; no explicit safety, regulatory, or stated primary-function loss applies to these DIRECT effects.</t>
+          <t>The End User effects tied directly to improper torque are noise (rattling/vibration) and potentially a cracked lamp; both are cosmetic/NVH issues and would be very objectionable to customers, aligning with Severity 4 per the table.</t>
         </is>
       </c>
       <c r="AP29" s="223" t="inlineStr">
         <is>
-          <t>Add in-station torque/angle monitoring with OK window and hard NOK gating (controller records each tightening and blocks completion if torque is below/above the 6 Nm spec).</t>
+          <t>Add in‑station electronic torque/angle monitoring with OK/NOK and data logging for each fastener (line stop on NOK) to catch under‑ or over‑torque events immediately.</t>
         </is>
       </c>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>Implement a DC transducerized torque tool with program lock tied to the headlamp barcode (6 Nm P-set) so only the correct tool/setting can run and it shuts off at target, preventing operator error, wrong tool use, and over‑/under‑torque.</t>
+          <t>Replace the current setup with a transducerized, programmable DC torque tool interlocked to the station (barcode/part ID selects the 6 Nm program and locks the tool if incorrect), eliminating wrong tool/setting use and operator over‑torque.</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Torque not achieved (under-torque); 2. Over torque. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED; 2. OVER TORQUE. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Test run_pipeline.py with merged-mode split-scoring wired in
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -2513,22 +2513,22 @@
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>The End User effects include 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation). With a merged mode 'SCRATCH / DAMAGE', the 'damage' sub-mode can directly yield a complete loss of headlamp function, mapping to Severity 8 per the table.</t>
+          <t>The End User effects explicitly state loss or degradation of the headlamp’s primary function (does not turn on; dim), with no safety-incident or regulatory language, so severity falls under primary function loss/degradation; given the merged 'scratch/damage' mode and unspecified 'damage,' both outcomes are plausible and the worst case (loss) is used.</t>
         </is>
       </c>
       <c r="AP18" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station camera-based vision inspection to automatically detect and reject headlamp lens/housing scratches or cracks before final tightening.</t>
+          <t>Install an inline automated vision inspection to detect lens/housing scratches and cracks after pick-and-connect, interlocked to stop the line on defect.</t>
         </is>
       </c>
       <c r="AQ18" s="223" t="inlineStr">
         <is>
-          <t>Add a pick-to-light bin-door interlock on the headlamp sequencing trolley tied to barcode scan and build manifest so the operator cannot access or select the wrong variant.</t>
+          <t>Replace the mixed storage trolley with keyed, foam-lined, one-slot-per-variant dunnage that physically segregates LH/RH and model variants to prevent part mix-up and contact damage during collection.</t>
         </is>
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it aligns with a 'wrong headlamp variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Merged failure mode: 1. SCRATCH; 2. DAMAGE ON HEAD LAMP. Scored separately: 'SCRATCH'=S7; 'DAMAGE ON HEAD LAMP'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage Mode; it aligns with a 'Wrong head lamp variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2630,22 +2630,22 @@
       </c>
       <c r="AN20" s="223" t="inlineStr">
         <is>
-          <t>The listed End User effects include both total loss of illumination and dim illumination. These map to loss or degradation of a primary vehicle function (headlighting). Without any explicit safety or regulatory wording, the worst-case direct outcome for the merged mode is "does not turn ON," which corresponds to S=8.</t>
+          <t>The End User effects list a primary-function failure: either the headlamp does not turn on (total loss) or is dim (degradation). No explicit safety or regulatory wording is present, so per the table this maps to Severity 8 (worst-case total loss of a primary vehicle function).</t>
         </is>
       </c>
       <c r="AP20" s="223" t="inlineStr">
         <is>
-          <t>Introduce an automated headlamp functional test at this station that commands ON and verifies illumination with a camera/lux sensor (or current sensor) before release.</t>
+          <t>Implement an automated power-on illumination test at this station using a light sensor/camera to verify the headlamp turns on and meets a minimum intensity threshold before release.</t>
         </is>
       </c>
       <c r="AQ20" s="223" t="inlineStr">
         <is>
-          <t>Add a VIN-linked pick-to-light/locking-bin system on the sequencing trolley so only the correct LH/RH headlamp bin illuminates and unlocks for the model, preventing wrong-part selection.</t>
+          <t>Add a model-specific locating/fastener-pattern go/no-go fixture that only allows the correct headlamp variant to seat and be torqued to 6 Nm, physically preventing installation of a wrong part.</t>
         </is>
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. FITMENT IS NOT FIRM; 2. WRONG SELECTION OF HEAD LAMP ( NOT AS PER MODEL). Scored separately: 'FITMENT IS NOT FIRM'=S8; 'WRONG SELECTION OF HEAD LAMP ( NOT AS PER MODEL)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2761,22 +2761,22 @@
       </c>
       <c r="AN22" s="223" t="inlineStr">
         <is>
-          <t>Improper/forgotten connector locking can leave the headlamp inoperative, which reduces road visibility; the End User effects explicitly state 'Increased risk of accident'. This matches the Severity 10 definition affecting safe vehicle operation and road user safety.</t>
+          <t>The End User effect explicitly lists 'Increased risk of accident', which is plausibly caused by an unconnected or improperly locked headlamp connector leading to no illumination or reduced visibility. This matches the Severity 10 definition for affecting safe operation/posing a safety risk to road users.</t>
         </is>
       </c>
       <c r="AP22" s="223" t="inlineStr">
         <is>
-          <t>Add an automated functional test at this station that powers the headlamp circuits and verifies current/illumination with a sensor, stopping the line if either connector is not making electrical contact.</t>
+          <t>Implement an automatic end-of-station headlamp functional test that commands the lamp ON and verifies current draw and/or light output with a sensor, with a hard go/no-go to stop the part if either connector is not providing illumination.</t>
         </is>
       </c>
       <c r="AQ22" s="223" t="inlineStr">
         <is>
-          <t>Install a keyed connector insertion fixture with a mechanical interlock that only releases the part for bolt tightening when both headlamp connectors are fully seated and latched to the hard-stop.</t>
+          <t>Add a connector-latch engagement poka-yoke (e.g., micro-switch/proximity sensor on each headlamp connector) that enables the bolt tool only when both connectors are fully locked, preventing the station from proceeding if a connector is forgotten or not latched.</t>
         </is>
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. Scored separately: 'IMPROPER LOCKING'=S10; 'POOR LOCKING'=S10. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2902,17 @@
       </c>
       <c r="AN24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly state 'Increased risk of accident', which is a safety consequence plausibly resulting from mis-aimed or non-functioning headlamps when bolts are not prefitted. Per the scoring rules, an explicit, causally plausible safety phrase requires Severity = 10.</t>
+          <t>The End User effects explicitly include 'Increased risk of accident,' which is a plausible outcome of a misaligned or non-functioning headlamp caused by missing prefit bolts, affecting safe operation of the vehicle. Per Table C2-1, this constitutes a safety/health risk to road users and requires Severity 10.</t>
         </is>
       </c>
       <c r="AP24" s="223" t="inlineStr">
         <is>
-          <t>Add an end-of-station vision check that verifies both headlamp bolts are present and seated (and lamp is flush/aligned), with NOK line stop and image traceability.</t>
+          <t>Install an automated vision check to verify both headlamp bolt heads are present and seated after assembly, triggering an NOK stop if either is missing.</t>
         </is>
       </c>
       <c r="AQ24" s="223" t="inlineStr">
         <is>
-          <t>Install a DC electric fastening system with controller that requires the required number of 6 Nm OK tighten events (bolt count) and locks out completion until achieved, with bolt-present/socket-present sensors on the tool.</t>
+          <t>Add a PLC-interlocked DC nutrunner that requires two OK torque–angle events at 6 Nm for the headlamp bolts before allowing station completion, preventing the operator from skipping the prefit step.</t>
         </is>
       </c>
       <c r="AR24" s="223" t="inlineStr">
@@ -3039,22 +3039,22 @@
       </c>
       <c r="AN26" s="223" t="inlineStr">
         <is>
-          <t>Among the listed End User effects, the direct outcome of missing/loose screws is rattling or vibration noise during driving, which maps to very objectionable sound/vibration per the table. More severe items like bulb burnout or water ingress require additional unstated failure mechanisms and are not used for the representative severity.</t>
+          <t>The most direct End User effect of missing fasteners or non-uniform gaps is 'rattling or vibration noise during driving,' which is an NVH issue; per the table this maps to 'Very objectionable ... sound, vibration,' giving Severity 4. Other listed effects (cracked lens, water ingress, burnout, eye strain) require additional unstated mechanisms and are indirect.</t>
         </is>
       </c>
       <c r="AP26" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station vision system to automatically measure headlamp-to-fender gap/flushness and verify both mounting screws are present/seated, interlocked to stop the line on fail.</t>
+          <t>Add a machine-vision check after installation to verify presence of all required screw heads and to measure/validate the perimeter gap at defined points with an interlock to stop the line on NOK.</t>
         </is>
       </c>
       <c r="AQ26" s="223" t="inlineStr">
         <is>
-          <t>Add a dedicated alignment/locator fixture with hard stops that sets the headlamp-to-fender gap uniformly and clamps the lamp in position during tightening so the operator cannot torque unless the gap is within spec.</t>
+          <t>Install a dedicated alignment/locator fixture with hard stops that positively locates the headlamp to the BIW to set the uniform gap before bolts are tightened, preventing the non-uniform-gap condition.</t>
         </is>
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap between headlamp and fender edge. Cause/Mode mismatch: The stated cause addresses only non-uniform gaps, not missing/failed-to-fit screws; it appears to belong to the 'not maintained gap' sub-mode rather than the 'failed to fit screws' sub-mode.</t>
+          <t>Merged failure mode: 1. Operator failed to fit screws; 2. Not maintained gap between headlamp and fender. Scored separately: 'Operator failed to fit screws'=S4; 'Not maintained gap between headlamp and fender'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: The stated cause addresses only non-uniform gaps and does not explain 'failed to fit screws'; scoring was based on the Mode text with worst-case among the merged sub-modes.</t>
         </is>
       </c>
     </row>
@@ -3183,17 +3183,17 @@
       </c>
       <c r="AN28" s="223" t="inlineStr">
         <is>
-          <t>Under‑torque leads to a loose headlamp mounting, which directly produces rattling/vibration noise during driving. This maps to "Very objectionable ... vibration/harshness" in the End User column. No explicit safety or regulatory effects are stated for this failure.</t>
+          <t>The direct customer-facing outcome of an under‑torqued headlamp mount is rattling/vibration noise during driving, which maps to very objectionable sound/vibration per the table. More severe effects listed (cracked lens, bulb burnout, water ingress) require additional unstated failure steps and are therefore not used to set severity.</t>
         </is>
       </c>
       <c r="AP28" s="223" t="inlineStr">
         <is>
-          <t>Add torque/angle monitoring with OK/NOK interlock on the tool so the station cannot release an OK until 6 Nm is achieved, with cycle‑by‑cycle traceable data logging.</t>
+          <t>Add an in-station torque/angle controller that records actual torque, provides OK/NOK with hard interlock to prevent workstation completion if 6 Nm is not achieved, and stores the torque trace to the VIN/part record.</t>
         </is>
       </c>
       <c r="AQ28" s="223" t="inlineStr">
         <is>
-          <t>Implement a controller‑locked DC torque tool preset to 6 Nm with station interlock (tool/spindle ID or RFID) so a wrong tool cannot run and the correct torque program is always applied.</t>
+          <t>Install a DC electric torque tool with programmed 6 Nm setpoint and tool-ID/station interlock so the wrong tool cannot be used and the fasteners cannot be completed unless target torque is reached.</t>
         </is>
       </c>
       <c r="AR28" s="223" t="inlineStr">
@@ -3246,22 +3246,22 @@
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
-          <t>The End User effects tied directly to improper torque are noise (rattling/vibration) and potentially a cracked lamp; both are cosmetic/NVH issues and would be very objectionable to customers, aligning with Severity 4 per the table.</t>
+          <t>For the torque-not-achieved/over-torque condition on headlamp mounting bolts, the only End User effect that follows directly is rattling/vibration noise during driving. This is an NVH complaint and is very objectionable, matching Severity 4. Other listed effects require additional unstated failure steps and are therefore indirect here.</t>
         </is>
       </c>
       <c r="AP29" s="223" t="inlineStr">
         <is>
-          <t>Add in‑station electronic torque/angle monitoring with OK/NOK and data logging for each fastener (line stop on NOK) to catch under‑ or over‑torque events immediately.</t>
+          <t>Add in-station electronic torque/angle monitoring with OK/NOK output and line stop for each fastener to verify 6 Nm is achieved within tolerance on 100% of parts.</t>
         </is>
       </c>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>Replace the current setup with a transducerized, programmable DC torque tool interlocked to the station (barcode/part ID selects the 6 Nm program and locks the tool if incorrect), eliminating wrong tool/setting use and operator over‑torque.</t>
+          <t>Replace the visually identified tool with a torque-controlled, shutoff nutrunner locked to 6 Nm via station interlock so the joint cannot be tightened with the wrong tool or outside the programmed torque.</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED; 2. OVER TORQUE. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. Torque not achieved (under-torque); 2. Over torque. Scored separately: 'Torque not achieved (under-torque)'=S4; 'Over torque'=S7. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild Excel with Sub-mode A/B columns from existing LLM data
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS29"/>
+  <dimension ref="A1:AY29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1622,7 +1622,13 @@
     <col width="8" customWidth="1" min="42" max="42"/>
     <col width="40" customWidth="1" min="43" max="43"/>
     <col width="45" customWidth="1" min="44" max="44"/>
-    <col width="60" customWidth="1" min="45" max="45"/>
+    <col width="30" customWidth="1" min="45" max="45"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="45" customWidth="1" min="47" max="47"/>
+    <col width="30" customWidth="1" min="48" max="48"/>
+    <col width="10" customWidth="1" min="49" max="49"/>
+    <col width="45" customWidth="1" min="50" max="50"/>
+    <col width="60" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2064,6 +2070,12 @@
       <c r="AQ13" s="205" t="n"/>
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
+      <c r="AT13" s="205" t="n"/>
+      <c r="AU13" s="205" t="n"/>
+      <c r="AV13" s="205" t="n"/>
+      <c r="AW13" s="205" t="n"/>
+      <c r="AX13" s="205" t="n"/>
+      <c r="AY13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2111,6 +2123,12 @@
       <c r="AQ14" s="205" t="n"/>
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
+      <c r="AT14" s="205" t="n"/>
+      <c r="AU14" s="205" t="n"/>
+      <c r="AV14" s="205" t="n"/>
+      <c r="AW14" s="205" t="n"/>
+      <c r="AX14" s="205" t="n"/>
+      <c r="AY14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2299,6 +2317,36 @@
         </is>
       </c>
       <c r="AS15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode A</t>
+        </is>
+      </c>
+      <c r="AT15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode A (S/D)</t>
+        </is>
+      </c>
+      <c r="AU15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode A Actions</t>
+        </is>
+      </c>
+      <c r="AV15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode B</t>
+        </is>
+      </c>
+      <c r="AW15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode B (S/D)</t>
+        </is>
+      </c>
+      <c r="AX15" s="208" t="inlineStr">
+        <is>
+          <t>Sub-mode B Actions</t>
+        </is>
+      </c>
+      <c r="AY15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -2350,6 +2398,12 @@
       <c r="AQ16" s="208" t="n"/>
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
+      <c r="AT16" s="208" t="n"/>
+      <c r="AU16" s="208" t="n"/>
+      <c r="AV16" s="208" t="n"/>
+      <c r="AW16" s="208" t="n"/>
+      <c r="AX16" s="208" t="n"/>
+      <c r="AY16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2397,6 +2451,12 @@
       <c r="AQ17" s="208" t="n"/>
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
+      <c r="AT17" s="208" t="n"/>
+      <c r="AU17" s="208" t="n"/>
+      <c r="AV17" s="208" t="n"/>
+      <c r="AW17" s="208" t="n"/>
+      <c r="AX17" s="208" t="n"/>
+      <c r="AY17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2523,25 +2583,55 @@
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>The End User effects list includes 'Headlamp does not turn ON', which is a total loss of the headlamp’s primary function; no explicit safety or regulatory wording is present, so this maps to Severity 8 per the table.</t>
-        </is>
-      </c>
-      <c r="AP18" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>The End User effects include 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation). With a merged mode 'SCRATCH / DAMAGE', the 'damage' sub-mode can directly yield a complete loss of headlamp function, mapping to Severity 8 per the table.</t>
+        </is>
+      </c>
+      <c r="AP18" s="223" t="n"/>
       <c r="AQ18" s="223" t="inlineStr">
         <is>
-          <t>Add an in-station machine-vision check for lens scratches/cracks with automatic reject/line-stop before installation.</t>
+          <t>Install an in-station camera-based vision inspection to automatically detect and reject headlamp lens/housing scratches or cracks before final tightening.</t>
         </is>
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>Install a pick-to-light system on the sequencing trolley with barcode/RFID scanner interlock to the station so only the VIN-correct headlamp bin can be picked and the process is locked out on any mismatch.</t>
+          <t>Add a pick-to-light bin-door interlock on the headlamp sequencing trolley tied to barcode scan and build manifest so the operator cannot access or select the wrong variant.</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Scored separately: 'Scratch on headlamp'=S4; 'Damage on headlamp'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Scratch on headlamp'=D8; 'Damage on headlamp'=D8. Per-mode actions: 'Scratch on headlamp': prevention - Add a barcode/RFID scan interlock at the pickup/installation step that compares the headlamp variant to the build manifest and disables tool enable/advancement if the wrong part is selected from the trolley.; detection - Install an in-station vision inspection with controlled lighting to automatically detect lens surface scratches and trigger an automatic reject before the unit leaves the station. | 'Damage on headlamp': prevention - Add a pick-to-light bin with barcode/RFID interlock that only enables access and unlocks the torque tool when the scanned headlamp part number matches the build manifest, preventing wrong-part selection from the storage trolley.; detection - Introduce an automated in-station headlamp functional test that powers the lamp and uses a sensor/camera to verify illumination and a minimum intensity threshold, blocking release on failure.. Cause/Mode mismatch: This Cause (wrong part selection/parts mix-up) does not inherently produce 'scratch/damage on headlamp' and reads like it belongs to a 'wrong variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Scratch on headlamp</t>
+        </is>
+      </c>
+      <c r="AT18" s="223" t="inlineStr">
+        <is>
+          <t>S4 / DNone</t>
+        </is>
+      </c>
+      <c r="AU18" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add individual soft-lined (foam/felt) pockets or separators to the sequencing/storage trolley so headlamps cannot contact each other or hard surfaces during handling, preventing scratches.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AV18" s="223" t="inlineStr">
+        <is>
+          <t>Damage on headlamp</t>
+        </is>
+      </c>
+      <c r="AW18" s="223" t="inlineStr">
+        <is>
+          <t>S8 / DNone</t>
+        </is>
+      </c>
+      <c r="AX18" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a pick-to-light and barcode-scan PLC interlock that only enables the torque tool when the scanned headlamp variant matches the build manifest for that VIN, preventing wrong-part selection from the storage trolley.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AY18" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Scored separately: 'Scratch on headlamp'=S4; 'Damage on headlamp'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Scratch on headlamp': prevention - Add individual soft-lined (foam/felt) pockets or separators to the sequencing/storage trolley so headlamps cannot contact each other or hard surfaces during handling, preventing scratches.; detection - n/a | 'Damage on headlamp': prevention - Add a pick-to-light and barcode-scan PLC interlock that only enables the torque tool when the scanned headlamp variant matches the build manifest for that VIN, preventing wrong-part selection from the storage trolley.; detection - n/a. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it aligns with a 'wrong headlamp variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2597,6 +2687,12 @@
       <c r="AQ19" s="223" t="n"/>
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
+      <c r="AT19" s="223" t="n"/>
+      <c r="AU19" s="223" t="n"/>
+      <c r="AV19" s="223" t="n"/>
+      <c r="AW19" s="223" t="n"/>
+      <c r="AX19" s="223" t="n"/>
+      <c r="AY19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2644,25 +2740,55 @@
       </c>
       <c r="AN20" s="223" t="inlineStr">
         <is>
-          <t>End User effects explicitly include loss/degradation of the headlamp’s primary function; with a wrong headlamp variant installed, 'does not turn ON' is a direct and plausible outcome, meeting the S=8 definition. No safety/accident wording or regulatory noncompliance is stated.</t>
-        </is>
-      </c>
-      <c r="AP20" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>The listed End User effects include both total loss of illumination and dim illumination. These map to loss or degradation of a primary vehicle function (headlighting). Without any explicit safety or regulatory wording, the worst-case direct outcome for the merged mode is "does not turn ON," which corresponds to S=8.</t>
+        </is>
+      </c>
+      <c r="AP20" s="223" t="n"/>
       <c r="AQ20" s="223" t="inlineStr">
         <is>
-          <t>Add an automated in-station headlamp functional test that powers the lamp and measures current/illuminance, stopping the station and blocking outflow on NOK.</t>
+          <t>Introduce an automated headlamp functional test at this station that commands ON and verifies illumination with a camera/lux sensor (or current sensor) before release.</t>
         </is>
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Add an interlocked barcode/RFID variant verification tied to the VIN/build sheet at the pick/scan step that prevents tool enablement or part release from the sequencing trolley if the scanned headlamp is not the correct model.</t>
+          <t>Add a VIN-linked pick-to-light/locking-bin system on the sequencing trolley so only the correct LH/RH headlamp bin illuminates and unlocks for the model, preventing wrong-part selection.</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. FITMENT IS NOT FIRM; 2. WRONG SELECTION OF HEAD LAMP (NOT AS PER MODEL). Scored separately: 'FITMENT IS NOT FIRM'=S8; 'WRONG SELECTION OF HEAD LAMP (NOT AS PER MODEL)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'FITMENT IS NOT FIRM'=D8; 'WRONG SELECTION OF HEAD LAMP (NOT AS PER MODEL)'=D8. Per-mode actions: 'FITMENT IS NOT FIRM': prevention - Add an interlocked barcode/RFID verification that compares the headlamp’s part number (LH/RH and variant) to the build manifest and prevents the torque tool from enabling if there is a mismatch.; detection - Add an automated in-station functional illumination test that powers the headlamp and measures light intensity/current to flag non-turn-on or dim-output parts before the unit leaves the station. | 'WRONG SELECTION OF HEAD LAMP (NOT AS PER MODEL)': prevention - Implement a VIN-linked pick-to-light/bin-locking system at the storage/POU so only the correct headlamp location illuminates/unlocks for the build and the wrong part cannot be picked.; detection - Add an automated in-station headlamp functional test that powers the unit and verifies ON/OFF and luminous flux against the model-specific spec with an automatic line stop on mismatch.. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Fitment is not firm</t>
+        </is>
+      </c>
+      <c r="AT20" s="223" t="inlineStr">
+        <is>
+          <t>S8 / DNone</t>
+        </is>
+      </c>
+      <c r="AU20" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a VIN-linked pick-to-light/locked-bin system on the sequencing trolley that only illuminates and unlocks the correct headlamp variant slot and prevents removal of any other part.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AV20" s="223" t="inlineStr">
+        <is>
+          <t>Wrong selection of head lamp (not as per model)</t>
+        </is>
+      </c>
+      <c r="AW20" s="223" t="inlineStr">
+        <is>
+          <t>S8 / DNone</t>
+        </is>
+      </c>
+      <c r="AX20" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Implement a pick-to-light bin system interlocked to the build record so only the correct headlamp variant bin illuminates/opens for each VIN, preventing wrong-part selection from the storage trolley.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AY20" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Scored separately: 'Fitment is not firm'=S8; 'Wrong selection of head lamp (not as per model)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Fitment is not firm': prevention - Add a VIN-linked pick-to-light/locked-bin system on the sequencing trolley that only illuminates and unlocks the correct headlamp variant slot and prevents removal of any other part.; detection - n/a | 'Wrong selection of head lamp (not as per model)': prevention - Implement a pick-to-light bin system interlocked to the build record so only the correct headlamp variant bin illuminates/opens for each VIN, preventing wrong-part selection from the storage trolley.; detection - n/a. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2716,6 +2842,12 @@
       <c r="AQ21" s="223" t="n"/>
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
+      <c r="AT21" s="223" t="n"/>
+      <c r="AU21" s="223" t="n"/>
+      <c r="AV21" s="223" t="n"/>
+      <c r="AW21" s="223" t="n"/>
+      <c r="AX21" s="223" t="n"/>
+      <c r="AY21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2779,23 +2911,27 @@
       </c>
       <c r="AN22" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include “Increased risk of accident,” which is a safety/health consequence that plausibly results from an unplugged/poorly locked headlamp connector leading to loss of lighting and reduced visibility. Per Table C2-1, this mandates Severity 10.</t>
-        </is>
-      </c>
-      <c r="AP22" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>Improper/forgotten connector locking can leave the headlamp inoperative, which reduces road visibility; the End User effects explicitly state 'Increased risk of accident'. This matches the Severity 10 definition affecting safe vehicle operation and road user safety.</t>
+        </is>
+      </c>
+      <c r="AP22" s="223" t="n"/>
       <c r="AQ22" s="223" t="inlineStr">
         <is>
-          <t>Implement an automated in-station headlamp functional test that powers the lamp and verifies current draw/illumination, with an interlock to stop the line or block advancement on fail.</t>
+          <t>Add an automated functional test at this station that powers the headlamp circuits and verifies current/illumination with a sensor, stopping the line if either connector is not making electrical contact.</t>
         </is>
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Add a connector insertion poka-yoke with force–travel monitoring that only releases/green-lights the step when both headlamp connectors are fully seated and latched, preventing progression if a connector is missed or partially engaged.</t>
-        </is>
-      </c>
-      <c r="AS22" s="223" t="inlineStr">
+          <t>Install a keyed connector insertion fixture with a mechanical interlock that only releases the part for bolt tightening when both headlamp connectors are fully seated and latched to the hard-stop.</t>
+        </is>
+      </c>
+      <c r="AS22" s="223" t="inlineStr"/>
+      <c r="AT22" s="223" t="inlineStr"/>
+      <c r="AU22" s="223" t="inlineStr"/>
+      <c r="AV22" s="223" t="inlineStr"/>
+      <c r="AW22" s="223" t="inlineStr"/>
+      <c r="AX22" s="223" t="inlineStr"/>
+      <c r="AY22" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2871,6 +3007,12 @@
       <c r="AQ23" s="223" t="n"/>
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
+      <c r="AT23" s="223" t="n"/>
+      <c r="AU23" s="223" t="n"/>
+      <c r="AV23" s="223" t="n"/>
+      <c r="AW23" s="223" t="n"/>
+      <c r="AX23" s="223" t="n"/>
+      <c r="AY23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -2924,23 +3066,27 @@
       </c>
       <c r="AN24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include “Increased risk of accident,” which is plausibly caused by a headlamp installed without prefitted bolts leading to misalignment and reduced visibility. Per the hard rule, an explicit accident risk on a lighting function requires Severity 10.</t>
-        </is>
-      </c>
-      <c r="AP24" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>The End User effects explicitly state 'Increased risk of accident', which is a safety consequence plausibly resulting from mis-aimed or non-functioning headlamps when bolts are not prefitted. Per the scoring rules, an explicit, causally plausible safety phrase requires Severity = 10.</t>
+        </is>
+      </c>
+      <c r="AP24" s="223" t="n"/>
       <c r="AQ24" s="223" t="inlineStr">
         <is>
-          <t>Install an in‑station automated bolt‑presence check (machine vision or inductive sensors) that verifies all required bolts are present and blocks station release if any are missing.</t>
+          <t>Add an end-of-station vision check that verifies both headlamp bolts are present and seated (and lamp is flush/aligned), with NOK line stop and image traceability.</t>
         </is>
       </c>
       <c r="AR24" s="223" t="inlineStr">
         <is>
-          <t>Add a bolt-presence poka‑yoke at this station (fixture/sensors that require all headlamp mounting bolts to be inserted before the torque tool enables or the station can advance).</t>
-        </is>
-      </c>
-      <c r="AS24" s="223" t="inlineStr">
+          <t>Install a DC electric fastening system with controller that requires the required number of 6 Nm OK tighten events (bolt count) and locks out completion until achieved, with bolt-present/socket-present sensors on the tool.</t>
+        </is>
+      </c>
+      <c r="AS24" s="223" t="inlineStr"/>
+      <c r="AT24" s="223" t="inlineStr"/>
+      <c r="AU24" s="223" t="inlineStr"/>
+      <c r="AV24" s="223" t="inlineStr"/>
+      <c r="AW24" s="223" t="inlineStr"/>
+      <c r="AX24" s="223" t="inlineStr"/>
+      <c r="AY24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -3000,6 +3146,12 @@
       <c r="AQ25" s="223" t="n"/>
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
+      <c r="AT25" s="223" t="n"/>
+      <c r="AU25" s="223" t="n"/>
+      <c r="AV25" s="223" t="n"/>
+      <c r="AW25" s="223" t="n"/>
+      <c r="AX25" s="223" t="n"/>
+      <c r="AY25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3065,25 +3217,55 @@
       </c>
       <c r="AN26" s="223" t="inlineStr">
         <is>
-          <t>Among the listed end user effects, only rattling/vibration noise follows directly from loose/missing screws and poor fit; this is a very objectionable NVH symptom, matching Severity 4. The other listed effects (cracked lens, bulb burnout, water ingress, eye strain) require additional unstated mechanisms and are therefore indirect for this mode/cause.</t>
-        </is>
-      </c>
-      <c r="AP26" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>Among the listed End User effects, the direct outcome of missing/loose screws is rattling or vibration noise during driving, which maps to very objectionable sound/vibration per the table. More severe items like bulb burnout or water ingress require additional unstated failure mechanisms and are not used for the representative severity.</t>
+        </is>
+      </c>
+      <c r="AP26" s="223" t="n"/>
       <c r="AQ26" s="223" t="inlineStr">
         <is>
-          <t>Add an in-station machine-vision check that verifies uniform gap around the headlamp perimeter and positively detects all screw heads present/seat condition before release.</t>
+          <t>Install an in-station vision system to automatically measure headlamp-to-fender gap/flushness and verify both mounting screws are present/seated, interlocked to stop the line on fail.</t>
         </is>
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Install a dedicated headlamp alignment/locating fixture with hard stops to set the design gap and clamp the lamp while tightening, combined with a screw-present interlock that prevents tool operation unless all screw positions are loaded.</t>
+          <t>Add a dedicated alignment/locator fixture with hard stops that sets the headlamp-to-fender gap uniformly and clamps the lamp in position during tightening so the operator cannot torque unless the gap is within spec.</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap. Scored separately: 'Failed to fit screws'=S4; 'Not maintained gap'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Failed to fit screws'=D8; 'Not maintained gap'=D8. Per-mode actions: 'Failed to fit screws': prevention - Add a dedicated headlamp alignment/locating fixture with datum pins/contoured nests to physically set uniform gaps and hold the lamp in position while the 6 Nm screws are started and torqued.; detection - Integrate torque–angle monitoring on the 6 Nm tool with OK/NOK interlock to automatically flag and stop release for under/over‑torque or cross‑thread conditions. | 'Not maintained gap': prevention - Install a dedicated in-station alignment fixture with hard locators/shims that set the headlamp-to-fender gap uniformly before the 6 Nm bolts can be torqued.; detection - Add an automated in-station vision/laser gap-and-flush measurement that blocks release if any measured gap point is out of specification.. Cause/Mode mismatch: The stated cause (operator doesn't maintain uniform gaps) aligns with the 'not maintained gap' sub-mode but does not explain the 'failed to fit screws' sub-mode, which would typically stem from a separate fastener-installation error.</t>
+          <t>Failed to fit screws</t>
+        </is>
+      </c>
+      <c r="AT26" s="223" t="inlineStr">
+        <is>
+          <t>S4 / DNone</t>
+        </is>
+      </c>
+      <c r="AU26" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a dedicated headlamp alignment/locator fixture with hard datums that sets the uniform gap to the fender and aligns the mounting holes so the screws can be installed without play or misposition.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AV26" s="223" t="inlineStr">
+        <is>
+          <t>Not maintained gap between headlamp and fender edge</t>
+        </is>
+      </c>
+      <c r="AW26" s="223" t="inlineStr">
+        <is>
+          <t>S4 / DNone</t>
+        </is>
+      </c>
+      <c r="AX26" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a simple alignment fixture with fixed datums and hard-stops that locates the headlamp relative to the fender edge before torquing to prevent non-uniform gaps.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AY26" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap between headlamp and fender edge. Scored separately: 'Failed to fit screws'=S4; 'Not maintained gap between headlamp and fender edge'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Failed to fit screws': prevention - Add a dedicated headlamp alignment/locator fixture with hard datums that sets the uniform gap to the fender and aligns the mounting holes so the screws can be installed without play or misposition.; detection - n/a | 'Not maintained gap between headlamp and fender edge': prevention - Add a simple alignment fixture with fixed datums and hard-stops that locates the headlamp relative to the fender edge before torquing to prevent non-uniform gaps.; detection - n/a. Cause/Mode mismatch: The stated cause addresses only non-uniform gaps, not missing/failed-to-fit screws; it appears to belong to the 'not maintained gap' sub-mode rather than the 'failed to fit screws' sub-mode.</t>
         </is>
       </c>
     </row>
@@ -3147,6 +3329,12 @@
       <c r="AQ27" s="223" t="n"/>
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
+      <c r="AT27" s="223" t="n"/>
+      <c r="AU27" s="223" t="n"/>
+      <c r="AV27" s="223" t="n"/>
+      <c r="AW27" s="223" t="n"/>
+      <c r="AX27" s="223" t="n"/>
+      <c r="AY27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3213,23 +3401,27 @@
       </c>
       <c r="AN28" s="223" t="inlineStr">
         <is>
-          <t>Under-torque at the headlamp mounting bolts most directly leads to a loose joint that rattles or vibrates during driving, which maps to very objectionable sound/vibration per the table (S=4). Other listed effects (lens crack, water ingress, bulb burnout) require additional unstated failure steps and are not used for severity scoring.</t>
-        </is>
-      </c>
-      <c r="AP28" s="223" t="n">
-        <v>9</v>
-      </c>
+          <t>Under‑torque leads to a loose headlamp mounting, which directly produces rattling/vibration noise during driving. This maps to "Very objectionable ... vibration/harshness" in the End User column. No explicit safety or regulatory effects are stated for this failure.</t>
+        </is>
+      </c>
+      <c r="AP28" s="223" t="n"/>
       <c r="AQ28" s="223" t="inlineStr">
         <is>
-          <t>Install a transducerized torque controller that records torque/angle for each fastener and provides in‑station OK/NOK with automatic line stop or reject if &lt;6 Nm.</t>
+          <t>Add torque/angle monitoring with OK/NOK interlock on the tool so the station cannot release an OK until 6 Nm is achieved, with cycle‑by‑cycle traceable data logging.</t>
         </is>
       </c>
       <c r="AR28" s="223" t="inlineStr">
         <is>
-          <t>Add RFID/tool-ID verification with controller lockout so only the correct, in-calibration power tool can run at this station, preventing wrong-tool use and use of out‑of‑calibration tools.</t>
-        </is>
-      </c>
-      <c r="AS28" s="223" t="inlineStr">
+          <t>Implement a controller‑locked DC torque tool preset to 6 Nm with station interlock (tool/spindle ID or RFID) so a wrong tool cannot run and the correct torque program is always applied.</t>
+        </is>
+      </c>
+      <c r="AS28" s="223" t="inlineStr"/>
+      <c r="AT28" s="223" t="inlineStr"/>
+      <c r="AU28" s="223" t="inlineStr"/>
+      <c r="AV28" s="223" t="inlineStr"/>
+      <c r="AW28" s="223" t="inlineStr"/>
+      <c r="AX28" s="223" t="inlineStr"/>
+      <c r="AY28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3279,56 +3471,95 @@
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
-          <t>The listed End User effects do not mention any accident/injury risk or regulatory noncompliance. The direct, representative outcomes of this torque error are cosmetic/NVH: a cracked/broken lens and rattling/vibration noise, both of which are very objectionable to customers, matching S=4.</t>
-        </is>
-      </c>
-      <c r="AP29" s="223" t="n">
-        <v>8</v>
-      </c>
+          <t>The End User effects tied directly to improper torque are noise (rattling/vibration) and potentially a cracked lamp; both are cosmetic/NVH issues and would be very objectionable to customers, aligning with Severity 4 per the table.</t>
+        </is>
+      </c>
+      <c r="AP29" s="223" t="n"/>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>Add in‑station torque/angle monitoring with a bolting controller that records achieved values per fastener and enforces an OK/NOK interlock so the station cannot complete if torque is out of specification.</t>
+          <t>Add in‑station electronic torque/angle monitoring with OK/NOK and data logging for each fastener (line stop on NOK) to catch under‑ or over‑torque events immediately.</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Upgrade to a transducerized, controller‑managed DC torque tool locked at 6 Nm with program/tool‑ID interlock and run‑inhibit on wrong tool or expired calibration to prevent under/over‑torque from operator error or mis‑calibration.</t>
+          <t>Replace the current setup with a transducerized, programmable DC torque tool interlocked to the station (barcode/part ID selects the 6 Nm program and locks the tool if incorrect), eliminating wrong tool/setting use and operator over‑torque.</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED (under-torque); 2. OVER TORQUE. Scored separately: 'TORQUE NOT ACHIEVED (under-torque)'=S4; 'OVER TORQUE'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'TORQUE NOT ACHIEVED (under-torque)'=D9; 'OVER TORQUE'=D9. Per-mode actions: 'TORQUE NOT ACHIEVED (under-torque)': prevention - Add a tool-controller interlock with RFID tool-ID and locked 6 Nm program that disables any non-approved tool and prevents operation if calibration status is expired.; detection - Install a transducerized DC fastening system that measures torque/angle for this joint with OK/NOK and line interlock to prevent progression until 6 Nm is achieved and recorded for 100% of parts. | 'OVER TORQUE': prevention - Install a DC torque‑controlled shut‑off nutrunner dedicated to this station, programmed to 6 Nm with an upper-limit lockout and tool-ID interlock to prevent use of the wrong or out‑of‑calibration tool.; detection - Add in‑station torque/angle monitoring with an OK/NOK window and automatic station interlock so any over‑torque event is flagged and the part cannot advance.. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>TORQUE NOT ACHIEVED</t>
+        </is>
+      </c>
+      <c r="AT29" s="223" t="inlineStr">
+        <is>
+          <t>S4 / DNone</t>
+        </is>
+      </c>
+      <c r="AU29" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Replace the current tool with a transducerized shut-off DC nutrunner preset to 6 Nm and interlocked to the station PLC so only the correct, calibrated program/tool can run and the cycle cannot complete unless the target torque is reached.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AV29" s="223" t="inlineStr">
+        <is>
+          <t>OVER TORQUE</t>
+        </is>
+      </c>
+      <c r="AW29" s="223" t="inlineStr">
+        <is>
+          <t>S4 / DNone</t>
+        </is>
+      </c>
+      <c r="AX29" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Replace the current tool with a DC torque-controlled nutrunner programmed to 6 Nm with an upper torque shut-off to prevent over-torque at this station.
+Detection: n/a</t>
+        </is>
+      </c>
+      <c r="AY29" s="223" t="inlineStr">
+        <is>
+          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED; 2. OVER TORQUE. Scored separately: 'TORQUE NOT ACHIEVED'=S4; 'OVER TORQUE'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'TORQUE NOT ACHIEVED': prevention - Replace the current tool with a transducerized shut-off DC nutrunner preset to 6 Nm and interlocked to the station PLC so only the correct, calibrated program/tool can run and the cycle cannot complete unless the target torque is reached.; detection - n/a | 'OVER TORQUE': prevention - Replace the current tool with a DC torque-controlled nutrunner programmed to 6 Nm with an upper torque shut-off to prevent over-torque at this station.; detection - n/a. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="163">
+  <mergeCells count="199">
     <mergeCell ref="AP18:AP19"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
+    <mergeCell ref="AT24:AT25"/>
     <mergeCell ref="AM15:AM17"/>
+    <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
+    <mergeCell ref="AV18:AV19"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
     <mergeCell ref="O23:O25"/>
+    <mergeCell ref="AT20:AT21"/>
     <mergeCell ref="M26:N29"/>
     <mergeCell ref="W15:X17"/>
     <mergeCell ref="T13:AA14"/>
     <mergeCell ref="S1:T2"/>
     <mergeCell ref="D12:F12"/>
+    <mergeCell ref="AU24:AU25"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G13:L14"/>
     <mergeCell ref="AR24:AR25"/>
     <mergeCell ref="K9:T9"/>
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
+    <mergeCell ref="AU26:AU27"/>
+    <mergeCell ref="AW26:AW27"/>
     <mergeCell ref="AN15:AN17"/>
+    <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
+    <mergeCell ref="AU18:AU19"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3341,6 +3572,7 @@
     <mergeCell ref="AP15:AP17"/>
     <mergeCell ref="K8:T8"/>
     <mergeCell ref="AR15:AR17"/>
+    <mergeCell ref="AY18:AY19"/>
     <mergeCell ref="Z23:Z25"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="M22:N25"/>
@@ -3348,13 +3580,18 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
+    <mergeCell ref="AT15:AT17"/>
+    <mergeCell ref="AV15:AV17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="AX15:AX17"/>
     <mergeCell ref="AN20:AN21"/>
     <mergeCell ref="AP20:AP21"/>
     <mergeCell ref="AQ22:AQ23"/>
     <mergeCell ref="AN26:AN27"/>
+    <mergeCell ref="AW24:AW25"/>
+    <mergeCell ref="AY24:AY25"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="R25:S25"/>
@@ -3362,6 +3599,7 @@
     <mergeCell ref="T25:U25"/>
     <mergeCell ref="AN22:AN23"/>
     <mergeCell ref="AP22:AP23"/>
+    <mergeCell ref="AY15:AY17"/>
     <mergeCell ref="P18:Q19"/>
     <mergeCell ref="AQ15:AQ17"/>
     <mergeCell ref="Y23:Y25"/>
@@ -3381,8 +3619,11 @@
     <mergeCell ref="AA15:AA17"/>
     <mergeCell ref="T22:U22"/>
     <mergeCell ref="AC15:AC17"/>
+    <mergeCell ref="AX20:AX21"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
+    <mergeCell ref="AV20:AV21"/>
+    <mergeCell ref="AX22:AX23"/>
     <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AS24:AS25"/>
     <mergeCell ref="AD15:AD17"/>
@@ -3394,12 +3635,13 @@
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
     <mergeCell ref="AS20:AS21"/>
+    <mergeCell ref="AU20:AU21"/>
     <mergeCell ref="AP24:AP25"/>
+    <mergeCell ref="AV22:AV23"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
     <mergeCell ref="G11:H11"/>
-    <mergeCell ref="AM13:AS14"/>
     <mergeCell ref="AH15:AH17"/>
     <mergeCell ref="AS22:AS23"/>
     <mergeCell ref="AJ15:AJ17"/>
@@ -3408,6 +3650,7 @@
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="O18:O21"/>
     <mergeCell ref="M18:N21"/>
+    <mergeCell ref="AY22:AY23"/>
     <mergeCell ref="AN18:AN19"/>
     <mergeCell ref="A1:R2"/>
     <mergeCell ref="AL15:AL17"/>
@@ -3417,11 +3660,18 @@
     <mergeCell ref="AM20:AM21"/>
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
+    <mergeCell ref="AV24:AV25"/>
+    <mergeCell ref="AX24:AX25"/>
+    <mergeCell ref="AX18:AX19"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
+    <mergeCell ref="AT22:AT23"/>
+    <mergeCell ref="AV26:AV27"/>
     <mergeCell ref="T19:U19"/>
+    <mergeCell ref="AU15:AU17"/>
+    <mergeCell ref="AW15:AW17"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
@@ -3430,16 +3680,19 @@
     <mergeCell ref="P29:Q29"/>
     <mergeCell ref="I15:J17"/>
     <mergeCell ref="C18:D29"/>
+    <mergeCell ref="AY26:AY27"/>
     <mergeCell ref="A15:B17"/>
     <mergeCell ref="K15:L17"/>
     <mergeCell ref="E18:F29"/>
     <mergeCell ref="W23:X27"/>
     <mergeCell ref="T20:U20"/>
+    <mergeCell ref="AM13:AY14"/>
     <mergeCell ref="I18:J21"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="Y27:Y29"/>
     <mergeCell ref="W18:X21"/>
     <mergeCell ref="K6:T6"/>
+    <mergeCell ref="AW18:AW19"/>
     <mergeCell ref="AB13:AL14"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="G10:H10"/>
@@ -3451,6 +3704,8 @@
     <mergeCell ref="Z15:Z17"/>
     <mergeCell ref="AQ18:AQ19"/>
     <mergeCell ref="AB15:AB17"/>
+    <mergeCell ref="AW20:AW21"/>
+    <mergeCell ref="AY20:AY21"/>
     <mergeCell ref="R21:S21"/>
     <mergeCell ref="T21:U21"/>
     <mergeCell ref="A10:C10"/>
@@ -3460,13 +3715,16 @@
     <mergeCell ref="Y15:Y17"/>
     <mergeCell ref="P26:Q27"/>
     <mergeCell ref="T26:U26"/>
+    <mergeCell ref="AW22:AW23"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="AU22:AU23"/>
     <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>
+    <mergeCell ref="AX26:AX27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Rebuild Excel with fresh Detection-per-split-mode data
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -2583,55 +2583,57 @@
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>The End User effects include 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation). With a merged mode 'SCRATCH / DAMAGE', the 'damage' sub-mode can directly yield a complete loss of headlamp function, mapping to Severity 8 per the table.</t>
-        </is>
-      </c>
-      <c r="AP18" s="223" t="n"/>
+          <t>The End User effects list includes "Headlamp does not turn ON" (total loss of the headlamp’s primary function) and "Insufficient brightness / dim light" (degradation). Per the table, total loss of a primary vehicle function maps to Severity 8; degradation would be 7, so worst-case for the merged Mode is 8.</t>
+        </is>
+      </c>
+      <c r="AP18" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ18" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station camera-based vision inspection to automatically detect and reject headlamp lens/housing scratches or cracks before final tightening.</t>
+          <t>Install an automated vision camera gate before bolt tightening to inspect the lens/housing for scratches or damage and automatically reject discrepant units.</t>
         </is>
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>Add a pick-to-light bin-door interlock on the headlamp sequencing trolley tied to barcode scan and build manifest so the operator cannot access or select the wrong variant.</t>
+          <t>Implement a barcode-scan interlock at the sequencing trolley pick point that only releases the part if the scanned part number matches the build VIN/model, preventing wrong-part selection/mix-up.</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>Scratch on headlamp</t>
+          <t>SCRATCH</t>
         </is>
       </c>
       <c r="AT18" s="223" t="inlineStr">
         <is>
-          <t>S4 / D(not scored - re-run needed)</t>
+          <t>S3 / D8</t>
         </is>
       </c>
       <c r="AU18" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add individual soft-lined (foam/felt) pockets or separators to the sequencing/storage trolley so headlamps cannot contact each other or hard surfaces during handling, preventing scratches.
-Detection: n/a</t>
+          <t>Prevention: Add variant-specific keyed bins/slots on the sequencing trolley with a scanner-interlocked pick-to-light that only releases the correct headlamp variant for the build, preventing wrong-part selection.
+Detection: Install an in-station automated vision inspection to check the headlamp lens surfaces for scratches before bolt tightening, with automatic reject on fail.</t>
         </is>
       </c>
       <c r="AV18" s="223" t="inlineStr">
         <is>
-          <t>Damage on headlamp</t>
+          <t>DAMAGE ON HEAD LAMP</t>
         </is>
       </c>
       <c r="AW18" s="223" t="inlineStr">
         <is>
-          <t>S8 / D(not scored - re-run needed)</t>
+          <t>S8 / D8</t>
         </is>
       </c>
       <c r="AX18" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add a pick-to-light and barcode-scan PLC interlock that only enables the torque tool when the scanned headlamp variant matches the build manifest for that VIN, preventing wrong-part selection from the storage trolley.
-Detection: n/a</t>
+          <t>Prevention: Add a pick-to-light with bin-lockout on the storage/sequence trolley tied to the build manifest so only the correct headlamp variant bin can be opened/picked, preventing wrong-part selection.
+Detection: Add an in-station automated functional light-on test with a photometric sensor that verifies each headlamp turns on and meets minimum intensity, interlocked to stop the process on fail.</t>
         </is>
       </c>
       <c r="AY18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Scratch on headlamp; 2. Damage on headlamp. Scored separately: 'Scratch on headlamp'=S4; 'Damage on headlamp'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Scratch on headlamp': prevention - Add individual soft-lined (foam/felt) pockets or separators to the sequencing/storage trolley so headlamps cannot contact each other or hard surfaces during handling, preventing scratches.; detection - n/a | 'Damage on headlamp': prevention - Add a pick-to-light and barcode-scan PLC interlock that only enables the torque tool when the scanned headlamp variant matches the build manifest for that VIN, preventing wrong-part selection from the storage trolley.; detection - n/a. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not physically produce a scratch/damage; it aligns with a 'wrong headlamp variant installed' failure mode instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Merged failure mode: 1. SCRATCH; 2. DAMAGE ON HEAD LAMP. Scored separately: 'SCRATCH'=S3; 'DAMAGE ON HEAD LAMP'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'SCRATCH'=D8; 'DAMAGE ON HEAD LAMP'=D8. Per-mode actions: 'SCRATCH': prevention - Add variant-specific keyed bins/slots on the sequencing trolley with a scanner-interlocked pick-to-light that only releases the correct headlamp variant for the build, preventing wrong-part selection.; detection - Install an in-station automated vision inspection to check the headlamp lens surfaces for scratches before bolt tightening, with automatic reject on fail. | 'DAMAGE ON HEAD LAMP': prevention - Add a pick-to-light with bin-lockout on the storage/sequence trolley tied to the build manifest so only the correct headlamp variant bin can be opened/picked, preventing wrong-part selection.; detection - Add an in-station automated functional light-on test with a photometric sensor that verifies each headlamp turns on and meets minimum intensity, interlocked to stop the process on fail.. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage Mode; it aligns with a 'wrong headlamp variant installed' failure instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2740,18 +2742,20 @@
       </c>
       <c r="AN20" s="223" t="inlineStr">
         <is>
-          <t>The listed End User effects include both total loss of illumination and dim illumination. These map to loss or degradation of a primary vehicle function (headlighting). Without any explicit safety or regulatory wording, the worst-case direct outcome for the merged mode is "does not turn ON," which corresponds to S=8.</t>
-        </is>
-      </c>
-      <c r="AP20" s="223" t="n"/>
+          <t>The End User effects list either a total loss of the headlamp’s primary function (does not turn ON) or a degradation (dim light); both are direct for the 'wrong selection of headlamp' sub-mode. Per the merged-mode worst-case rule, the total loss case maps to S=8.</t>
+        </is>
+      </c>
+      <c r="AP20" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ20" s="223" t="inlineStr">
         <is>
-          <t>Introduce an automated headlamp functional test at this station that commands ON and verifies illumination with a camera/lux sensor (or current sensor) before release.</t>
+          <t>Add an automated in-station power-on test with current/photometric verification and interlock that blocks release if the headlamp fails to turn on or is below the expected threshold.</t>
         </is>
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Add a VIN-linked pick-to-light/locking-bin system on the sequencing trolley so only the correct LH/RH headlamp bin illuminates and unlocks for the model, preventing wrong-part selection.</t>
+          <t>Add a VIN/model-linked pick-to-light system with bin-locking on the sequencing trolley so only the correct headlamp variant bin illuminates/unlocks, preventing the operator from picking a wrong part.</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
@@ -2761,34 +2765,34 @@
       </c>
       <c r="AT20" s="223" t="inlineStr">
         <is>
-          <t>S8 / D(not scored - re-run needed)</t>
+          <t>S8 / D8</t>
         </is>
       </c>
       <c r="AU20" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add a VIN-linked pick-to-light/locked-bin system on the sequencing trolley that only illuminates and unlocks the correct headlamp variant slot and prevents removal of any other part.
-Detection: n/a</t>
+          <t>Prevention: Add a barcode/RFID variant verification interlock that only enables the 6 Nm torque tool (OK-to-bolt) when the scanned headlamp PN matches the vehicle build spec, preventing wrong-part installation from the sequencing trolley.
+Detection: Introduce an automated in-station headlamp functional/photometric test that powers the lamp and measures ON status and minimum brightness, with a hard stop if requirements are not met.</t>
         </is>
       </c>
       <c r="AV20" s="223" t="inlineStr">
         <is>
-          <t>Wrong selection of head lamp (not as per model)</t>
+          <t>Wrong selection of headlamp (not as per model)</t>
         </is>
       </c>
       <c r="AW20" s="223" t="inlineStr">
         <is>
-          <t>S8 / D(not scored - re-run needed)</t>
+          <t>S8 / D7</t>
         </is>
       </c>
       <c r="AX20" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Implement a pick-to-light bin system interlocked to the build record so only the correct headlamp variant bin illuminates/opens for each VIN, preventing wrong-part selection from the storage trolley.
-Detection: n/a</t>
+          <t>Prevention: Add a pick-to-light with bin lockout at the sequencing trolley keyed to the vehicle VIN/model so only the correct headlamp part number can be released for the job and access to other bins is physically blocked.
+Detection: Install an in-station automated barcode/OCR verification of the installed headlamp part label against the build record with a hard line stop/torque-gun lockout on any mismatch.</t>
         </is>
       </c>
       <c r="AY20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of head lamp (not as per model). Scored separately: 'Fitment is not firm'=S8; 'Wrong selection of head lamp (not as per model)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Fitment is not firm': prevention - Add a VIN-linked pick-to-light/locked-bin system on the sequencing trolley that only illuminates and unlocks the correct headlamp variant slot and prevents removal of any other part.; detection - n/a | 'Wrong selection of head lamp (not as per model)': prevention - Implement a pick-to-light bin system interlocked to the build record so only the correct headlamp variant bin illuminates/opens for each VIN, preventing wrong-part selection from the storage trolley.; detection - n/a. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of headlamp (not as per model). Scored separately: 'Fitment is not firm'=S8; 'Wrong selection of headlamp (not as per model)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Fitment is not firm'=D8; 'Wrong selection of headlamp (not as per model)'=D7. Per-mode actions: 'Fitment is not firm': prevention - Add a barcode/RFID variant verification interlock that only enables the 6 Nm torque tool (OK-to-bolt) when the scanned headlamp PN matches the vehicle build spec, preventing wrong-part installation from the sequencing trolley.; detection - Introduce an automated in-station headlamp functional/photometric test that powers the lamp and measures ON status and minimum brightness, with a hard stop if requirements are not met. | 'Wrong selection of headlamp (not as per model)': prevention - Add a pick-to-light with bin lockout at the sequencing trolley keyed to the vehicle VIN/model so only the correct headlamp part number can be released for the job and access to other bins is physically blocked.; detection - Install an in-station automated barcode/OCR verification of the installed headlamp part label against the build record with a hard line stop/torque-gun lockout on any mismatch.. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2911,29 +2915,57 @@
       </c>
       <c r="AN22" s="223" t="inlineStr">
         <is>
-          <t>Improper/forgotten connector locking can leave the headlamp inoperative, which reduces road visibility; the End User effects explicitly state 'Increased risk of accident'. This matches the Severity 10 definition affecting safe vehicle operation and road user safety.</t>
-        </is>
-      </c>
-      <c r="AP22" s="223" t="n"/>
+          <t>Improper/poor locking of the headlamp electrical connectors can leave the lamp non-functional, leading to reduced road visibility and the explicitly stated "increased risk of accident" for the end user. The AIAG‑VDA table assigns such safety/accident risk to Severity 10.</t>
+        </is>
+      </c>
+      <c r="AP22" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ22" s="223" t="inlineStr">
         <is>
-          <t>Add an automated functional test at this station that powers the headlamp circuits and verifies current/illumination with a sensor, stopping the line if either connector is not making electrical contact.</t>
+          <t>Add an automated end‑of‑station functional test that powers the headlamp and verifies illumination/current draw for required circuits, with automatic line stop on fail.</t>
         </is>
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Install a keyed connector insertion fixture with a mechanical interlock that only releases the part for bolt tightening when both headlamp connectors are fully seated and latched to the hard-stop.</t>
-        </is>
-      </c>
-      <c r="AS22" s="223" t="inlineStr"/>
-      <c r="AT22" s="223" t="inlineStr"/>
-      <c r="AU22" s="223" t="inlineStr"/>
-      <c r="AV22" s="223" t="inlineStr"/>
-      <c r="AW22" s="223" t="inlineStr"/>
-      <c r="AX22" s="223" t="inlineStr"/>
+          <t>Add an interlocked connector-seating poka‑yoke with stroke/force sensing that only enables the bolt‑tightening tool after both headlamp connectors are fully latched (positive lock detected).</t>
+        </is>
+      </c>
+      <c r="AS22" s="223" t="inlineStr">
+        <is>
+          <t>IMPROPER LOCKING</t>
+        </is>
+      </c>
+      <c r="AT22" s="223" t="inlineStr">
+        <is>
+          <t>S10 / D8</t>
+        </is>
+      </c>
+      <c r="AU22" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a poka‑yoke latch-position/CPA presence sensor on each headlamp connector interlocked to enable the torque tool only when both connectors are fully seated and locked.
+Detection: Add an automated in-station headlamp functional test that powers the lamp and verifies current/illumination with a sensor, blocking release if either connector is not properly seated.</t>
+        </is>
+      </c>
+      <c r="AV22" s="223" t="inlineStr">
+        <is>
+          <t>POOR LOCKING</t>
+        </is>
+      </c>
+      <c r="AW22" s="223" t="inlineStr">
+        <is>
+          <t>S10 / D8</t>
+        </is>
+      </c>
+      <c r="AX22" s="223" t="inlineStr">
+        <is>
+          <t>Prevention: Add a connector-latch poka‑yoke interlock (latch presence/seat sensor tied to the station) that prevents proceeding to bolt‑tightening until both headlamp connectors are fully seated and latched.
+Detection: Install an automated in‑station functional test that powers the headlamp and verifies illumination/continuity for each connector with an interlocked pass/fail gate that stops the part if either side fails.</t>
+        </is>
+      </c>
       <c r="AY22" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. Scored separately: 'IMPROPER LOCKING'=S10; 'POOR LOCKING'=S10. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'IMPROPER LOCKING'=D8; 'POOR LOCKING'=D8. Per-mode actions: 'IMPROPER LOCKING': prevention - Add a poka‑yoke latch-position/CPA presence sensor on each headlamp connector interlocked to enable the torque tool only when both connectors are fully seated and locked.; detection - Add an automated in-station headlamp functional test that powers the lamp and verifies current/illumination with a sensor, blocking release if either connector is not properly seated. | 'POOR LOCKING': prevention - Add a connector-latch poka‑yoke interlock (latch presence/seat sensor tied to the station) that prevents proceeding to bolt‑tightening until both headlamp connectors are fully seated and latched.; detection - Install an automated in‑station functional test that powers the headlamp and verifies illumination/continuity for each connector with an interlocked pass/fail gate that stops the part if either side fails.. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -3066,18 +3098,20 @@
       </c>
       <c r="AN24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly state 'Increased risk of accident', which is a safety consequence plausibly resulting from mis-aimed or non-functioning headlamps when bolts are not prefitted. Per the scoring rules, an explicit, causally plausible safety phrase requires Severity = 10.</t>
-        </is>
-      </c>
-      <c r="AP24" s="223" t="n"/>
+          <t>The End User effects explicitly include "Increased risk of accident," which is a plausible consequence of missing prefit bolts causing misalignment or non-function leading to reduced road visibility. Per the scoring rules, an explicit safety consequence requires Severity 10.</t>
+        </is>
+      </c>
+      <c r="AP24" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ24" s="223" t="inlineStr">
         <is>
-          <t>Add an end-of-station vision check that verifies both headlamp bolts are present and seated (and lamp is flush/aligned), with NOK line stop and image traceability.</t>
+          <t>Add a machine-based bolt presence and torque/angle verification (vision or prox sensors confirming both bolt heads plus DC tool signature) with station interlock that stops the line if any headlamp prefit bolt is missing.</t>
         </is>
       </c>
       <c r="AR24" s="223" t="inlineStr">
         <is>
-          <t>Install a DC electric fastening system with controller that requires the required number of 6 Nm OK tighten events (bolt count) and locks out completion until achieved, with bolt-present/socket-present sensors on the tool.</t>
+          <t>Install an in-station bolt-present poka‑yoke (pick-to-light with count verification plus bolt-start presence sensors) that prevents advancing the job until all required headlamp prefit bolts are inserted.</t>
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr"/>
@@ -3217,55 +3251,57 @@
       </c>
       <c r="AN26" s="223" t="inlineStr">
         <is>
-          <t>Among the listed End User effects, the direct outcome of missing/loose screws is rattling or vibration noise during driving, which maps to very objectionable sound/vibration per the table. More severe items like bulb burnout or water ingress require additional unstated failure mechanisms and are not used for the representative severity.</t>
-        </is>
-      </c>
-      <c r="AP26" s="223" t="n"/>
+          <t>Among the listed End User effects, only rattling/vibration noise follows directly from missing/under-installed screws and improper gap; it is an NVH/cosmetic issue and aligns with the table’s “very objectionable … sound, vibration” definition.</t>
+        </is>
+      </c>
+      <c r="AP26" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ26" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station vision system to automatically measure headlamp-to-fender gap/flushness and verify both mounting screws are present/seated, interlocked to stop the line on fail.</t>
+          <t>Install an in-station machine-vision check to measure headlamp-to-fender gaps at multiple points and confirm all mounting screws are present after torque, with automatic line stop on fail.</t>
         </is>
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Add a dedicated alignment/locator fixture with hard stops that sets the headlamp-to-fender gap uniformly and clamps the lamp in position during tightening so the operator cannot torque unless the gap is within spec.</t>
+          <t>Add a headlamp alignment/locating fixture with hard datum stops that set the lamp-to-fender gap before tightening, preventing fastening unless the lamp is seated to the locators (poka‑yoke for uniform gaps).</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>Failed to fit screws</t>
+          <t>FAILED TO FIT SCREWS</t>
         </is>
       </c>
       <c r="AT26" s="223" t="inlineStr">
         <is>
-          <t>S4 / D(not scored - re-run needed)</t>
+          <t>S4 / D8</t>
         </is>
       </c>
       <c r="AU26" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add a dedicated headlamp alignment/locator fixture with hard datums that sets the uniform gap to the fender and aligns the mounting holes so the screws can be installed without play or misposition.
-Detection: n/a</t>
+          <t>Prevention: Install a headlamp alignment/locating fixture with datum pins and hard gap shims that hold the lamp to the BIW at the specified uniform gaps so the screw holes are aligned before tightening.
+Detection: Add a DC electric screwdriver with torque–angle monitoring and screw-count interlock (or a vision screw-present check) that prevents station completion if any required mounting screw is missing.</t>
         </is>
       </c>
       <c r="AV26" s="223" t="inlineStr">
         <is>
-          <t>Not maintained gap between headlamp and fender edge</t>
+          <t>NOT MAINTAINED GAP</t>
         </is>
       </c>
       <c r="AW26" s="223" t="inlineStr">
         <is>
-          <t>S4 / D(not scored - re-run needed)</t>
+          <t>S4 / D8</t>
         </is>
       </c>
       <c r="AX26" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add a simple alignment fixture with fixed datums and hard-stops that locates the headlamp relative to the fender edge before torquing to prevent non-uniform gaps.
-Detection: n/a</t>
+          <t>Prevention: Add a simple alignment/locating fixture with hard stops that sets the headlamp-to-fender gap uniformly before torquing so the operator cannot tighten bolts unless the lamp is seated to the specified flushness.
+Detection: Install an in-station camera or laser gap/flush measurement system that automatically measures the headlamp–fender gap around the perimeter and stops the line or flags a reject if limits are exceeded.</t>
         </is>
       </c>
       <c r="AY26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. Failed to fit screws; 2. Not maintained gap between headlamp and fender edge. Scored separately: 'Failed to fit screws'=S4; 'Not maintained gap between headlamp and fender edge'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'Failed to fit screws': prevention - Add a dedicated headlamp alignment/locator fixture with hard datums that sets the uniform gap to the fender and aligns the mounting holes so the screws can be installed without play or misposition.; detection - n/a | 'Not maintained gap between headlamp and fender edge': prevention - Add a simple alignment fixture with fixed datums and hard-stops that locates the headlamp relative to the fender edge before torquing to prevent non-uniform gaps.; detection - n/a. Cause/Mode mismatch: The stated cause addresses only non-uniform gaps, not missing/failed-to-fit screws; it appears to belong to the 'not maintained gap' sub-mode rather than the 'failed to fit screws' sub-mode.</t>
+          <t>Merged failure mode: 1. FAILED TO FIT SCREWS; 2. NOT MAINTAINED GAP. Scored separately: 'FAILED TO FIT SCREWS'=S4; 'NOT MAINTAINED GAP'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'FAILED TO FIT SCREWS'=D8; 'NOT MAINTAINED GAP'=D8. Per-mode actions: 'FAILED TO FIT SCREWS': prevention - Install a headlamp alignment/locating fixture with datum pins and hard gap shims that hold the lamp to the BIW at the specified uniform gaps so the screw holes are aligned before tightening.; detection - Add a DC electric screwdriver with torque–angle monitoring and screw-count interlock (or a vision screw-present check) that prevents station completion if any required mounting screw is missing. | 'NOT MAINTAINED GAP': prevention - Add a simple alignment/locating fixture with hard stops that sets the headlamp-to-fender gap uniformly before torquing so the operator cannot tighten bolts unless the lamp is seated to the specified flushness.; detection - Install an in-station camera or laser gap/flush measurement system that automatically measures the headlamp–fender gap around the perimeter and stops the line or flags a reject if limits are exceeded..</t>
         </is>
       </c>
     </row>
@@ -3401,18 +3437,20 @@
       </c>
       <c r="AN28" s="223" t="inlineStr">
         <is>
-          <t>Under‑torque leads to a loose headlamp mounting, which directly produces rattling/vibration noise during driving. This maps to "Very objectionable ... vibration/harshness" in the End User column. No explicit safety or regulatory effects are stated for this failure.</t>
-        </is>
-      </c>
-      <c r="AP28" s="223" t="n"/>
+          <t>Under-torque of the headlamp mounting bolts most directly causes rattling/vibration noise during driving, which fits the 'very objectionable' NVH category. No explicit accident/injury or regulatory noncompliance effect is stated for this mode, and the primary lighting function loss effects listed are indirect.</t>
+        </is>
+      </c>
+      <c r="AP28" s="223" t="n">
+        <v>8</v>
+      </c>
       <c r="AQ28" s="223" t="inlineStr">
         <is>
-          <t>Add torque/angle monitoring with OK/NOK interlock on the tool so the station cannot release an OK until 6 Nm is achieved, with cycle‑by‑cycle traceable data logging.</t>
+          <t>Implement a transducerized DC nutrunner (torque/angle logging) with bolt count and OK/NOK interlock that blocks station completion if 6 Nm is not achieved.</t>
         </is>
       </c>
       <c r="AR28" s="223" t="inlineStr">
         <is>
-          <t>Implement a controller‑locked DC torque tool preset to 6 Nm with station interlock (tool/spindle ID or RFID) so a wrong tool cannot run and the correct torque program is always applied.</t>
+          <t>Add RFID/tool-parameter lockout and socket/bit coding so only the correct, calibrated tool with the 6 Nm program can be used at this station, preventing operator error and wrong-tool use.</t>
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr"/>
@@ -3471,55 +3509,57 @@
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
-          <t>The End User effects tied directly to improper torque are noise (rattling/vibration) and potentially a cracked lamp; both are cosmetic/NVH issues and would be very objectionable to customers, aligning with Severity 4 per the table.</t>
-        </is>
-      </c>
-      <c r="AP29" s="223" t="n"/>
+          <t>The End User effects directly tied to incorrect torque are rattling/vibration noise and visible cracking, both of which are very objectionable to customers and align with the S4 definition; no safety or regulatory language is present, and no explicit loss/degradation of the primary lighting function is stated.</t>
+        </is>
+      </c>
+      <c r="AP29" s="223" t="n">
+        <v>9</v>
+      </c>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>Add in‑station electronic torque/angle monitoring with OK/NOK and data logging for each fastener (line stop on NOK) to catch under‑ or over‑torque events immediately.</t>
+          <t>Add in-station torque/angle monitoring with an OK/NOK controller that records achieved values per fastener and stops the line or flags NOK if the 6 Nm spec is not met.</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Replace the current setup with a transducerized, programmable DC torque tool interlocked to the station (barcode/part ID selects the 6 Nm program and locks the tool if incorrect), eliminating wrong tool/setting use and operator over‑torque.</t>
+          <t>Install a DC torque/angle-controlled nutrunner locked to the 6 Nm specification via part barcode scan with controller interlock to prevent completion if torque is out of spec, eliminating wrong-tool use and over/under-torque from operator error or mis-calibration.</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>TORQUE NOT ACHIEVED</t>
+          <t>Torque not achieved (under-torque)</t>
         </is>
       </c>
       <c r="AT29" s="223" t="inlineStr">
         <is>
-          <t>S4 / D(not scored - re-run needed)</t>
+          <t>S4 / D8</t>
         </is>
       </c>
       <c r="AU29" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Replace the current tool with a transducerized shut-off DC nutrunner preset to 6 Nm and interlocked to the station PLC so only the correct, calibrated program/tool can run and the cycle cannot complete unless the target torque is reached.
-Detection: n/a</t>
+          <t>Prevention: Replace the station’s driver with a controller‑based shutoff (transducerized) torque tool locked to 6 Nm for this joint to error‑proof operator technique and wrong‑tool use.
+Detection: Add 100% in‑station torque/angle verification with the tool’s OK/NOK interlock that prevents process completion/release if any fastener is below spec.</t>
         </is>
       </c>
       <c r="AV29" s="223" t="inlineStr">
         <is>
-          <t>OVER TORQUE</t>
+          <t>Over torque</t>
         </is>
       </c>
       <c r="AW29" s="223" t="inlineStr">
         <is>
-          <t>S4 / D(not scored - re-run needed)</t>
+          <t>S4 / D9</t>
         </is>
       </c>
       <c r="AX29" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Replace the current tool with a DC torque-controlled nutrunner programmed to 6 Nm with an upper torque shut-off to prevent over-torque at this station.
-Detection: n/a</t>
+          <t>Prevention: Replace the current tool with a transducerized, torque-controlled driver locked to a 6 Nm window with an upper-limit shutoff and PLC interlock so over‑torque cannot be applied.
+Detection: Add in-station torque monitoring/trace capture with programmed upper/lower limits and automatic NOK line stop if torque exceeds the upper limit.</t>
         </is>
       </c>
       <c r="AY29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode: 1. TORQUE NOT ACHIEVED; 2. OVER TORQUE. Scored separately: 'TORQUE NOT ACHIEVED'=S4; 'OVER TORQUE'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Per-mode actions: 'TORQUE NOT ACHIEVED': prevention - Replace the current tool with a transducerized shut-off DC nutrunner preset to 6 Nm and interlocked to the station PLC so only the correct, calibrated program/tool can run and the cycle cannot complete unless the target torque is reached.; detection - n/a | 'OVER TORQUE': prevention - Replace the current tool with a DC torque-controlled nutrunner programmed to 6 Nm with an upper torque shut-off to prevent over-torque at this station.; detection - n/a. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode: 1. Torque not achieved (under-torque); 2. Over torque. Scored separately: 'Torque not achieved (under-torque)'=S4; 'Over torque'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Torque not achieved (under-torque)'=D8; 'Over torque'=D9. Per-mode actions: 'Torque not achieved (under-torque)': prevention - Replace the station’s driver with a controller‑based shutoff (transducerized) torque tool locked to 6 Nm for this joint to error‑proof operator technique and wrong‑tool use.; detection - Add 100% in‑station torque/angle verification with the tool’s OK/NOK interlock that prevents process completion/release if any fastener is below spec. | 'Over torque': prevention - Replace the current tool with a transducerized, torque-controlled driver locked to a 6 Nm window with an upper-limit shutoff and PLC interlock so over‑torque cannot be applied.; detection - Add in-station torque monitoring/trace capture with programmed upper/lower limits and automatic NOK line stop if torque exceeds the upper limit.. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fresh run with cause/mode mismatch override for actions
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions.xlsx
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY29"/>
+  <dimension ref="A1:AV29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1622,13 +1622,10 @@
     <col width="8" customWidth="1" min="42" max="42"/>
     <col width="40" customWidth="1" min="43" max="43"/>
     <col width="45" customWidth="1" min="44" max="44"/>
-    <col width="30" customWidth="1" min="45" max="45"/>
-    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="35" customWidth="1" min="45" max="45"/>
+    <col width="45" customWidth="1" min="46" max="46"/>
     <col width="45" customWidth="1" min="47" max="47"/>
-    <col width="30" customWidth="1" min="48" max="48"/>
-    <col width="10" customWidth="1" min="49" max="49"/>
-    <col width="45" customWidth="1" min="50" max="50"/>
-    <col width="60" customWidth="1" min="51" max="51"/>
+    <col width="50" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2073,9 +2070,6 @@
       <c r="AT13" s="205" t="n"/>
       <c r="AU13" s="205" t="n"/>
       <c r="AV13" s="205" t="n"/>
-      <c r="AW13" s="205" t="n"/>
-      <c r="AX13" s="205" t="n"/>
-      <c r="AY13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2126,9 +2120,6 @@
       <c r="AT14" s="205" t="n"/>
       <c r="AU14" s="205" t="n"/>
       <c r="AV14" s="205" t="n"/>
-      <c r="AW14" s="205" t="n"/>
-      <c r="AX14" s="205" t="n"/>
-      <c r="AY14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2318,35 +2309,20 @@
       </c>
       <c r="AS15" s="208" t="inlineStr">
         <is>
-          <t>Sub-mode A</t>
+          <t>Sub-modes</t>
         </is>
       </c>
       <c r="AT15" s="208" t="inlineStr">
         <is>
-          <t>Sub-mode A (S/D)</t>
+          <t>Sub-mode Prevention</t>
         </is>
       </c>
       <c r="AU15" s="208" t="inlineStr">
         <is>
-          <t>Sub-mode A Actions</t>
+          <t>Sub-mode Detection</t>
         </is>
       </c>
       <c r="AV15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-mode B</t>
-        </is>
-      </c>
-      <c r="AW15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-mode B (S/D)</t>
-        </is>
-      </c>
-      <c r="AX15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-mode B Actions</t>
-        </is>
-      </c>
-      <c r="AY15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -2401,9 +2377,6 @@
       <c r="AT16" s="208" t="n"/>
       <c r="AU16" s="208" t="n"/>
       <c r="AV16" s="208" t="n"/>
-      <c r="AW16" s="208" t="n"/>
-      <c r="AX16" s="208" t="n"/>
-      <c r="AY16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2454,9 +2427,6 @@
       <c r="AT17" s="208" t="n"/>
       <c r="AU17" s="208" t="n"/>
       <c r="AV17" s="208" t="n"/>
-      <c r="AW17" s="208" t="n"/>
-      <c r="AX17" s="208" t="n"/>
-      <c r="AY17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2583,7 +2553,7 @@
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>The End User effects list includes "Headlamp does not turn ON" (total loss of the headlamp’s primary function) and "Insufficient brightness / dim light" (degradation). Per the table, total loss of a primary vehicle function maps to Severity 8; degradation would be 7, so worst-case for the merged Mode is 8.</t>
+          <t>The End User effects list includes 'Headlamp does not turn ON', which is a total loss of the headlamp’s primary lighting function; no safety/accident wording or regulatory noncompliance is stated, so S=8 per the table.</t>
         </is>
       </c>
       <c r="AP18" s="223" t="n">
@@ -2591,49 +2561,35 @@
       </c>
       <c r="AQ18" s="223" t="inlineStr">
         <is>
-          <t>Install an automated vision camera gate before bolt tightening to inspect the lens/housing for scratches or damage and automatically reject discrepant units.</t>
+          <t>Add an in-station machine-vision inspection with controlled lighting to detect lens scratches/damage and interlock the station to reject the headlamp on defect detection.</t>
         </is>
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>Implement a barcode-scan interlock at the sequencing trolley pick point that only releases the part if the scanned part number matches the build VIN/model, preventing wrong-part selection/mix-up.</t>
+          <t>The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: add soft-lined, dedicated headlamp nests and protective lens films/caps on parts and trolleys to prevent contact with hard edges during handling and alignment.</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>SCRATCH</t>
+          <t>A = Scratch on headlamp (S7/D8)
+B = Damage on headlamp (S8/D8)</t>
         </is>
       </c>
       <c r="AT18" s="223" t="inlineStr">
         <is>
-          <t>S3 / D8</t>
+          <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: apply a removable protective film to the headlamp lens from storage through installation, with a poka‑yoke removal step at final inspection to prevent handling scratches.
+B = The plant's recorded Cause does not match this Mode; addressing the more plausible damage mechanism instead: add a padded alignment/installation fixture with hard locating stops to support the headlamp and prevent lens/housing contact with the BIW during fitment and tightening.</t>
         </is>
       </c>
       <c r="AU18" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add variant-specific keyed bins/slots on the sequencing trolley with a scanner-interlocked pick-to-light that only releases the correct headlamp variant for the build, preventing wrong-part selection.
-Detection: Install an in-station automated vision inspection to check the headlamp lens surfaces for scratches before bolt tightening, with automatic reject on fail.</t>
+          <t>A = Add a machine‑vision inspection with controlled lighting to detect lens scratches and interlock the station to automatically reject discrepant headlamps.
+B = Add an in-station automated functional illumination test that powers the headlamp and measures current and lux with go/no-go limits to catch 'does not turn ON' and 'dim' before release.</t>
         </is>
       </c>
       <c r="AV18" s="223" t="inlineStr">
         <is>
-          <t>DAMAGE ON HEAD LAMP</t>
-        </is>
-      </c>
-      <c r="AW18" s="223" t="inlineStr">
-        <is>
-          <t>S8 / D8</t>
-        </is>
-      </c>
-      <c r="AX18" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Add a pick-to-light with bin-lockout on the storage/sequence trolley tied to the build manifest so only the correct headlamp variant bin can be opened/picked, preventing wrong-part selection.
-Detection: Add an in-station automated functional light-on test with a photometric sensor that verifies each headlamp turns on and meets minimum intensity, interlocked to stop the process on fail.</t>
-        </is>
-      </c>
-      <c r="AY18" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. SCRATCH; 2. DAMAGE ON HEAD LAMP. Scored separately: 'SCRATCH'=S3; 'DAMAGE ON HEAD LAMP'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'SCRATCH'=D8; 'DAMAGE ON HEAD LAMP'=D8. Per-mode actions: 'SCRATCH': prevention - Add variant-specific keyed bins/slots on the sequencing trolley with a scanner-interlocked pick-to-light that only releases the correct headlamp variant for the build, preventing wrong-part selection.; detection - Install an in-station automated vision inspection to check the headlamp lens surfaces for scratches before bolt tightening, with automatic reject on fail. | 'DAMAGE ON HEAD LAMP': prevention - Add a pick-to-light with bin-lockout on the storage/sequence trolley tied to the build manifest so only the correct headlamp variant bin can be opened/picked, preventing wrong-part selection.; detection - Add an in-station automated functional light-on test with a photometric sensor that verifies each headlamp turns on and meets minimum intensity, interlocked to stop the process on fail.. Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage Mode; it aligns with a 'wrong headlamp variant installed' failure instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2692,9 +2648,6 @@
       <c r="AT19" s="223" t="n"/>
       <c r="AU19" s="223" t="n"/>
       <c r="AV19" s="223" t="n"/>
-      <c r="AW19" s="223" t="n"/>
-      <c r="AX19" s="223" t="n"/>
-      <c r="AY19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2742,7 +2695,7 @@
       </c>
       <c r="AN20" s="223" t="inlineStr">
         <is>
-          <t>The End User effects list either a total loss of the headlamp’s primary function (does not turn ON) or a degradation (dim light); both are direct for the 'wrong selection of headlamp' sub-mode. Per the merged-mode worst-case rule, the total loss case maps to S=8.</t>
+          <t>The End User effects list includes both total loss (does not turn ON) and degradation (dim light) of the headlamp’s primary function; no safety or regulatory wording is present. Using the worst-case direct outcome for wrong-part selection yields Severity 8.</t>
         </is>
       </c>
       <c r="AP20" s="223" t="n">
@@ -2750,49 +2703,35 @@
       </c>
       <c r="AQ20" s="223" t="inlineStr">
         <is>
-          <t>Add an automated in-station power-on test with current/photometric verification and interlock that blocks release if the headlamp fails to turn on or is below the expected threshold.</t>
+          <t>Install a camera-based vision check that reads the headlamp’s model/label and interlocks the station (no bolt enable) if the variant does not match the VIN/build record.</t>
         </is>
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Add a VIN/model-linked pick-to-light system with bin-locking on the sequencing trolley so only the correct headlamp variant bin illuminates/unlocks, preventing the operator from picking a wrong part.</t>
+          <t>Add VIN-driven bin lockout on the headlamp sequencing trolley so only the correct headlamp variant bin opens for the current vehicle, preventing wrong-part selection at pickup.</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
         <is>
-          <t>Fitment is not firm</t>
+          <t>A = Fitment is not firm (S8/D8)
+B = Wrong selection of headlamp (not as per model) (S8/D8)</t>
         </is>
       </c>
       <c r="AT20" s="223" t="inlineStr">
         <is>
-          <t>S8 / D8</t>
+          <t>A = Add a VIN-driven pick-to-light/scan-interlocked sequencing trolley that only enables the correct headlamp bin for the build and alarms/locks the process if any other bin is accessed to prevent wrong-part picks.
+B = Add a barcode/RFID scan interlock tied to the build manifest that only enables the torque tool and allows installation when the scanned headlamp part number matches the vehicle model at this station.</t>
         </is>
       </c>
       <c r="AU20" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Add a barcode/RFID variant verification interlock that only enables the 6 Nm torque tool (OK-to-bolt) when the scanned headlamp PN matches the vehicle build spec, preventing wrong-part installation from the sequencing trolley.
-Detection: Introduce an automated in-station headlamp functional/photometric test that powers the lamp and measures ON status and minimum brightness, with a hard stop if requirements are not met.</t>
+          <t>A = Use an in-station DC torque tool with transducer and PLC OK/NOK lockout to verify 6 Nm on each headlamp fastener and prevent release if torque is not achieved (detecting non-firm fitment).
+B = Implement an automated in-station headlamp functional test that powers the lamp after connection and measures current/illumination with sensors, stopping the line and flagging a mismatch if the unit is off or out of spec.</t>
         </is>
       </c>
       <c r="AV20" s="223" t="inlineStr">
         <is>
-          <t>Wrong selection of headlamp (not as per model)</t>
-        </is>
-      </c>
-      <c r="AW20" s="223" t="inlineStr">
-        <is>
-          <t>S8 / D7</t>
-        </is>
-      </c>
-      <c r="AX20" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Add a pick-to-light with bin lockout at the sequencing trolley keyed to the vehicle VIN/model so only the correct headlamp part number can be released for the job and access to other bins is physically blocked.
-Detection: Install an in-station automated barcode/OCR verification of the installed headlamp part label against the build record with a hard line stop/torque-gun lockout on any mismatch.</t>
-        </is>
-      </c>
-      <c r="AY20" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Fitment is not firm; 2. Wrong selection of headlamp (not as per model). Scored separately: 'Fitment is not firm'=S8; 'Wrong selection of headlamp (not as per model)'=S8. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Fitment is not firm'=D8; 'Wrong selection of headlamp (not as per model)'=D7. Per-mode actions: 'Fitment is not firm': prevention - Add a barcode/RFID variant verification interlock that only enables the 6 Nm torque tool (OK-to-bolt) when the scanned headlamp PN matches the vehicle build spec, preventing wrong-part installation from the sequencing trolley.; detection - Introduce an automated in-station headlamp functional/photometric test that powers the lamp and measures ON status and minimum brightness, with a hard stop if requirements are not met. | 'Wrong selection of headlamp (not as per model)': prevention - Add a pick-to-light with bin lockout at the sequencing trolley keyed to the vehicle VIN/model so only the correct headlamp part number can be released for the job and access to other bins is physically blocked.; detection - Install an in-station automated barcode/OCR verification of the installed headlamp part label against the build record with a hard line stop/torque-gun lockout on any mismatch.. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2849,9 +2788,6 @@
       <c r="AT21" s="223" t="n"/>
       <c r="AU21" s="223" t="n"/>
       <c r="AV21" s="223" t="n"/>
-      <c r="AW21" s="223" t="n"/>
-      <c r="AX21" s="223" t="n"/>
-      <c r="AY21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2915,7 +2851,7 @@
       </c>
       <c r="AN22" s="223" t="inlineStr">
         <is>
-          <t>Improper/poor locking of the headlamp electrical connectors can leave the lamp non-functional, leading to reduced road visibility and the explicitly stated "increased risk of accident" for the end user. The AIAG‑VDA table assigns such safety/accident risk to Severity 10.</t>
+          <t>The End User effects explicitly list 'Increased risk of accident', which is causally plausible for an unconnected/poorly locked headlamp connector causing the lamp not to turn on and reducing visibility. Per the table, this is a safety/health risk to road users, so Severity is 10.</t>
         </is>
       </c>
       <c r="AP22" s="223" t="n">
@@ -2923,49 +2859,20 @@
       </c>
       <c r="AQ22" s="223" t="inlineStr">
         <is>
-          <t>Add an automated end‑of‑station functional test that powers the headlamp and verifies illumination/current draw for required circuits, with automatic line stop on fail.</t>
+          <t>Add an in‑station automated functional test that powers each headlamp and verifies illumination/current draw with a light or current sensor, stopping the process if either lamp fails.</t>
         </is>
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Add an interlocked connector-seating poka‑yoke with stroke/force sensing that only enables the bolt‑tightening tool after both headlamp connectors are fully latched (positive lock detected).</t>
-        </is>
-      </c>
-      <c r="AS22" s="223" t="inlineStr">
-        <is>
-          <t>IMPROPER LOCKING</t>
-        </is>
-      </c>
-      <c r="AT22" s="223" t="inlineStr">
-        <is>
-          <t>S10 / D8</t>
-        </is>
-      </c>
-      <c r="AU22" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Add a poka‑yoke latch-position/CPA presence sensor on each headlamp connector interlocked to enable the torque tool only when both connectors are fully seated and locked.
-Detection: Add an automated in-station headlamp functional test that powers the lamp and verifies current/illumination with a sensor, blocking release if either connector is not properly seated.</t>
-        </is>
-      </c>
+          <t>Add a connector-lock poka‑yoke: a mechanical go/no‑go gauge or latch‑position sensor interlocked with the station PLC so the cycle cannot complete unless the connector latch is fully engaged.</t>
+        </is>
+      </c>
+      <c r="AS22" s="223" t="inlineStr"/>
+      <c r="AT22" s="223" t="inlineStr"/>
+      <c r="AU22" s="223" t="inlineStr"/>
       <c r="AV22" s="223" t="inlineStr">
         <is>
-          <t>POOR LOCKING</t>
-        </is>
-      </c>
-      <c r="AW22" s="223" t="inlineStr">
-        <is>
-          <t>S10 / D8</t>
-        </is>
-      </c>
-      <c r="AX22" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Add a connector-latch poka‑yoke interlock (latch presence/seat sensor tied to the station) that prevents proceeding to bolt‑tightening until both headlamp connectors are fully seated and latched.
-Detection: Install an automated in‑station functional test that powers the headlamp and verifies illumination/continuity for each connector with an interlocked pass/fail gate that stops the part if either side fails.</t>
-        </is>
-      </c>
-      <c r="AY22" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. IMPROPER LOCKING; 2. POOR LOCKING. Scored separately: 'IMPROPER LOCKING'=S10; 'POOR LOCKING'=S10. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'IMPROPER LOCKING'=D8; 'POOR LOCKING'=D8. Per-mode actions: 'IMPROPER LOCKING': prevention - Add a poka‑yoke latch-position/CPA presence sensor on each headlamp connector interlocked to enable the torque tool only when both connectors are fully seated and locked.; detection - Add an automated in-station headlamp functional test that powers the lamp and verifies current/illumination with a sensor, blocking release if either connector is not properly seated. | 'POOR LOCKING': prevention - Add a connector-latch poka‑yoke interlock (latch presence/seat sensor tied to the station) that prevents proceeding to bolt‑tightening until both headlamp connectors are fully seated and latched.; detection - Install an automated in‑station functional test that powers the headlamp and verifies illumination/continuity for each connector with an interlocked pass/fail gate that stops the part if either side fails.. AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
     </row>
@@ -3042,9 +2949,6 @@
       <c r="AT23" s="223" t="n"/>
       <c r="AU23" s="223" t="n"/>
       <c r="AV23" s="223" t="n"/>
-      <c r="AW23" s="223" t="n"/>
-      <c r="AX23" s="223" t="n"/>
-      <c r="AY23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -3098,7 +3002,7 @@
       </c>
       <c r="AN24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include "Increased risk of accident," which is a plausible consequence of missing prefit bolts causing misalignment or non-function leading to reduced road visibility. Per the scoring rules, an explicit safety consequence requires Severity 10.</t>
+          <t>The End User effects explicitly state 'Increased risk of accident,' which is a plausible consequence of an unbolted/misaligned headlamp causing reduced road illumination. Per the scoring rules and Table C2-1, this constitutes an effect that affects safe operation of the vehicle, warranting Severity 10.</t>
         </is>
       </c>
       <c r="AP24" s="223" t="n">
@@ -3106,21 +3010,18 @@
       </c>
       <c r="AQ24" s="223" t="inlineStr">
         <is>
-          <t>Add a machine-based bolt presence and torque/angle verification (vision or prox sensors confirming both bolt heads plus DC tool signature) with station interlock that stops the line if any headlamp prefit bolt is missing.</t>
+          <t>Install a machine-vision presence/position check at station exit to verify both headlamp bolt heads are present and seated, with automatic NOK stop/reject if either bolt is missing.</t>
         </is>
       </c>
       <c r="AR24" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station bolt-present poka‑yoke (pick-to-light with count verification plus bolt-start presence sensors) that prevents advancing the job until all required headlamp prefit bolts are inserted.</t>
+          <t>Add a DC electric nutrunner with torque/angle monitoring and an OK-to-proceed interlock that requires both headlamp bolts to be run to 6 Nm (correct count and torque achieved) before allowing the station to complete.</t>
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr"/>
       <c r="AT24" s="223" t="inlineStr"/>
       <c r="AU24" s="223" t="inlineStr"/>
-      <c r="AV24" s="223" t="inlineStr"/>
-      <c r="AW24" s="223" t="inlineStr"/>
-      <c r="AX24" s="223" t="inlineStr"/>
-      <c r="AY24" s="223" t="inlineStr">
+      <c r="AV24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -3183,9 +3084,6 @@
       <c r="AT25" s="223" t="n"/>
       <c r="AU25" s="223" t="n"/>
       <c r="AV25" s="223" t="n"/>
-      <c r="AW25" s="223" t="n"/>
-      <c r="AX25" s="223" t="n"/>
-      <c r="AY25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3251,7 +3149,7 @@
       </c>
       <c r="AN26" s="223" t="inlineStr">
         <is>
-          <t>Among the listed End User effects, only rattling/vibration noise follows directly from missing/under-installed screws and improper gap; it is an NVH/cosmetic issue and aligns with the table’s “very objectionable … sound, vibration” definition.</t>
+          <t>Among the listed End User effects, only "Rattling or vibration noise during driving" follows directly from missing/loose screws or poor fit. This is an NVH complaint that customers would find very objectionable, matching the table’s description for Severity 4.</t>
         </is>
       </c>
       <c r="AP26" s="223" t="n">
@@ -3259,49 +3157,35 @@
       </c>
       <c r="AQ26" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station machine-vision check to measure headlamp-to-fender gaps at multiple points and confirm all mounting screws are present after torque, with automatic line stop on fail.</t>
+          <t>Install an in-station machine-vision check that verifies all headlamp screw presence and measures the headlamp–fender gap against limits, stopping the station on NG.</t>
         </is>
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Add a headlamp alignment/locating fixture with hard datum stops that set the lamp-to-fender gap before tightening, preventing fastening unless the lamp is seated to the locators (poka‑yoke for uniform gaps).</t>
+          <t>Add a pin-locating/stop fixture to set the headlamp-to-fender gap and a torque tool with screw-count and 6 Nm OK interlock that prevents job completion if any headlamp screw is missing or out of spec.</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>FAILED TO FIT SCREWS</t>
+          <t>A = Failed to fit screws (S4/D8)
+B = Not maintained gap (S4/D8)</t>
         </is>
       </c>
       <c r="AT26" s="223" t="inlineStr">
         <is>
-          <t>S4 / D8</t>
+          <t>A = Add a datum-based alignment/locator fixture with hard edge stops and hole locators to set the headlamp-to-fender gap and align the screw bosses before fastening so screws can be fitted correctly every time.
+B = Add a dedicated locating/positioning fixture or hard datum pins at the headlamp mounting points to set flushness and gap to spec before torquing, preventing misalignment by design.</t>
         </is>
       </c>
       <c r="AU26" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Install a headlamp alignment/locating fixture with datum pins and hard gap shims that hold the lamp to the BIW at the specified uniform gaps so the screw holes are aligned before tightening.
-Detection: Add a DC electric screwdriver with torque–angle monitoring and screw-count interlock (or a vision screw-present check) that prevents station completion if any required mounting screw is missing.</t>
+          <t>A = Use an electronic torque controller that counts each fastener and verifies torque/angle OK for all required screws, blocking proceed on any missing/under/over-torqued condition.
+B = Install an in-station camera-based gap/flushness measurement system interlocked to the station (block OK-to-release if any measured gap/flushness is out of spec).</t>
         </is>
       </c>
       <c r="AV26" s="223" t="inlineStr">
         <is>
-          <t>NOT MAINTAINED GAP</t>
-        </is>
-      </c>
-      <c r="AW26" s="223" t="inlineStr">
-        <is>
-          <t>S4 / D8</t>
-        </is>
-      </c>
-      <c r="AX26" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Add a simple alignment/locating fixture with hard stops that sets the headlamp-to-fender gap uniformly before torquing so the operator cannot tighten bolts unless the lamp is seated to the specified flushness.
-Detection: Install an in-station camera or laser gap/flush measurement system that automatically measures the headlamp–fender gap around the perimeter and stops the line or flags a reject if limits are exceeded.</t>
-        </is>
-      </c>
-      <c r="AY26" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. FAILED TO FIT SCREWS; 2. NOT MAINTAINED GAP. Scored separately: 'FAILED TO FIT SCREWS'=S4; 'NOT MAINTAINED GAP'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'FAILED TO FIT SCREWS'=D8; 'NOT MAINTAINED GAP'=D8. Per-mode actions: 'FAILED TO FIT SCREWS': prevention - Install a headlamp alignment/locating fixture with datum pins and hard gap shims that hold the lamp to the BIW at the specified uniform gaps so the screw holes are aligned before tightening.; detection - Add a DC electric screwdriver with torque–angle monitoring and screw-count interlock (or a vision screw-present check) that prevents station completion if any required mounting screw is missing. | 'NOT MAINTAINED GAP': prevention - Add a simple alignment/locating fixture with hard stops that sets the headlamp-to-fender gap uniformly before torquing so the operator cannot tighten bolts unless the lamp is seated to the specified flushness.; detection - Install an in-station camera or laser gap/flush measurement system that automatically measures the headlamp–fender gap around the perimeter and stops the line or flags a reject if limits are exceeded..</t>
+          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
         </is>
       </c>
     </row>
@@ -3368,9 +3252,6 @@
       <c r="AT27" s="223" t="n"/>
       <c r="AU27" s="223" t="n"/>
       <c r="AV27" s="223" t="n"/>
-      <c r="AW27" s="223" t="n"/>
-      <c r="AX27" s="223" t="n"/>
-      <c r="AY27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3437,29 +3318,26 @@
       </c>
       <c r="AN28" s="223" t="inlineStr">
         <is>
-          <t>Under-torque of the headlamp mounting bolts most directly causes rattling/vibration noise during driving, which fits the 'very objectionable' NVH category. No explicit accident/injury or regulatory noncompliance effect is stated for this mode, and the primary lighting function loss effects listed are indirect.</t>
+          <t>The only direct customer effect of an under-torqued headlamp mounting is rattling/vibration noise while driving, which is an NVH issue. The list contains no explicit safety or regulatory consequence tied to this mode, so severity aligns with "very objectionable" NVH at S=4.</t>
         </is>
       </c>
       <c r="AP28" s="223" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AQ28" s="223" t="inlineStr">
         <is>
-          <t>Implement a transducerized DC nutrunner (torque/angle logging) with bolt count and OK/NOK interlock that blocks station completion if 6 Nm is not achieved.</t>
+          <t>Install a transducerized DC nutrunner or in-line torque/angle monitor that records actual achieved torque and provides OK/NOK with line stop if 6 Nm is not reached.</t>
         </is>
       </c>
       <c r="AR28" s="223" t="inlineStr">
         <is>
-          <t>Add RFID/tool-parameter lockout and socket/bit coding so only the correct, calibrated tool with the 6 Nm program can be used at this station, preventing operator error and wrong-tool use.</t>
+          <t>Add a station interlock with tool-ID/torque-program lock (RFID/barcode pairing) so only the correct, calibrated 6 Nm power tool can run this joint and its torque setting cannot be changed by the operator.</t>
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr"/>
       <c r="AT28" s="223" t="inlineStr"/>
       <c r="AU28" s="223" t="inlineStr"/>
-      <c r="AV28" s="223" t="inlineStr"/>
-      <c r="AW28" s="223" t="inlineStr"/>
-      <c r="AX28" s="223" t="inlineStr"/>
-      <c r="AY28" s="223" t="inlineStr">
+      <c r="AV28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3509,7 +3387,7 @@
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
-          <t>The End User effects directly tied to incorrect torque are rattling/vibration noise and visible cracking, both of which are very objectionable to customers and align with the S4 definition; no safety or regulatory language is present, and no explicit loss/degradation of the primary lighting function is stated.</t>
+          <t>The only direct End User outcome of a torque error on the headlamp mounting fasteners is NVH (rattling/vibration noise during driving). No explicit accident/injury or regulatory noncompliance is stated, and loss of lighting function is only listed via indirect effects. NVH that customers would clearly notice maps to Severity 4.</t>
         </is>
       </c>
       <c r="AP29" s="223" t="n">
@@ -3517,55 +3395,41 @@
       </c>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>Add in-station torque/angle monitoring with an OK/NOK controller that records achieved values per fastener and stops the line or flags NOK if the 6 Nm spec is not met.</t>
+          <t>Add in‑station electronic torque verification that records torque/angle for each bolt and issues an automatic NOK/stop if any rundown is outside the 6 Nm window before the unit can leave the station.</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Install a DC torque/angle-controlled nutrunner locked to the 6 Nm specification via part barcode scan with controller interlock to prevent completion if torque is out of spec, eliminating wrong-tool use and over/under-torque from operator error or mis-calibration.</t>
+          <t>Replace the current setup with a DC electric torque tool locked at 6 Nm with torque/angle control and socket/tool-ID poka‑yoke to prevent wrong tool use and eliminate operator-set errors.</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>Torque not achieved (under-torque)</t>
+          <t>A = Torque not achieved (S4/D9)
+B = Over torque (S4/D9)</t>
         </is>
       </c>
       <c r="AT29" s="223" t="inlineStr">
         <is>
-          <t>S4 / D8</t>
+          <t>A = Install a DC electric nutrunner with controller‑locked 6 Nm program and RFID/tool‑ID lockout so the station cannot run with the wrong tool or setting, directly addressing operator mistake and wrong/miscalibrated tool causes.
+B = Install a DC torque-controlled driver locked to a 6 Nm window with OK/NOK lockout (paired to this station/tool ID) to prevent over‑torque from operator error, wrong tool use, or drift.</t>
         </is>
       </c>
       <c r="AU29" s="223" t="inlineStr">
         <is>
-          <t>Prevention: Replace the station’s driver with a controller‑based shutoff (transducerized) torque tool locked to 6 Nm for this joint to error‑proof operator technique and wrong‑tool use.
-Detection: Add 100% in‑station torque/angle verification with the tool’s OK/NOK interlock that prevents process completion/release if any fastener is below spec.</t>
+          <t>A = Integrate in‑station torque monitoring (nutrunner torque‑angle OK/NOK with PLC interlock) so the station cannot advance unless each fastener achieves the 6 Nm OK result.
+B = Integrate in‑station electronic torque monitoring with data logging and an interlock that blocks job release if the recorded torque is outside the 6 Nm window (OK/NOK confirmation).</t>
         </is>
       </c>
       <c r="AV29" s="223" t="inlineStr">
         <is>
-          <t>Over torque</t>
-        </is>
-      </c>
-      <c r="AW29" s="223" t="inlineStr">
-        <is>
-          <t>S4 / D9</t>
-        </is>
-      </c>
-      <c r="AX29" s="223" t="inlineStr">
-        <is>
-          <t>Prevention: Replace the current tool with a transducerized, torque-controlled driver locked to a 6 Nm window with an upper-limit shutoff and PLC interlock so over‑torque cannot be applied.
-Detection: Add in-station torque monitoring/trace capture with programmed upper/lower limits and automatic NOK line stop if torque exceeds the upper limit.</t>
-        </is>
-      </c>
-      <c r="AY29" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode: 1. Torque not achieved (under-torque); 2. Over torque. Scored separately: 'Torque not achieved (under-torque)'=S4; 'Over torque'=S4. Row-level Severity above is the worst case; consider splitting this row in the plant sheet. Detection per mode: 'Torque not achieved (under-torque)'=D8; 'Over torque'=D9. Per-mode actions: 'Torque not achieved (under-torque)': prevention - Replace the station’s driver with a controller‑based shutoff (transducerized) torque tool locked to 6 Nm for this joint to error‑proof operator technique and wrong‑tool use.; detection - Add 100% in‑station torque/angle verification with the tool’s OK/NOK interlock that prevents process completion/release if any fastener is below spec. | 'Over torque': prevention - Replace the current tool with a transducerized, torque-controlled driver locked to a 6 Nm window with an upper-limit shutoff and PLC interlock so over‑torque cannot be applied.; detection - Add in-station torque monitoring/trace capture with programmed upper/lower limits and automatic NOK line stop if torque exceeds the upper limit.. Ambiguous - plausible severities: S4 (Lens cracked or broken); S4 (Rattling or vibration noise during driving). Suggested value is the worst case; review before finalizing. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="199">
+  <mergeCells count="181">
     <mergeCell ref="AP18:AP19"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
@@ -3593,7 +3457,6 @@
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
     <mergeCell ref="AU26:AU27"/>
-    <mergeCell ref="AW26:AW27"/>
     <mergeCell ref="AN15:AN17"/>
     <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
@@ -3612,7 +3475,6 @@
     <mergeCell ref="AP15:AP17"/>
     <mergeCell ref="K8:T8"/>
     <mergeCell ref="AR15:AR17"/>
-    <mergeCell ref="AY18:AY19"/>
     <mergeCell ref="Z23:Z25"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="M22:N25"/>
@@ -3620,18 +3482,16 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
+    <mergeCell ref="AM13:AV14"/>
     <mergeCell ref="AT15:AT17"/>
     <mergeCell ref="AV15:AV17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="AX15:AX17"/>
     <mergeCell ref="AN20:AN21"/>
     <mergeCell ref="AP20:AP21"/>
     <mergeCell ref="AQ22:AQ23"/>
     <mergeCell ref="AN26:AN27"/>
-    <mergeCell ref="AW24:AW25"/>
-    <mergeCell ref="AY24:AY25"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="R25:S25"/>
@@ -3639,7 +3499,6 @@
     <mergeCell ref="T25:U25"/>
     <mergeCell ref="AN22:AN23"/>
     <mergeCell ref="AP22:AP23"/>
-    <mergeCell ref="AY15:AY17"/>
     <mergeCell ref="P18:Q19"/>
     <mergeCell ref="AQ15:AQ17"/>
     <mergeCell ref="Y23:Y25"/>
@@ -3659,11 +3518,9 @@
     <mergeCell ref="AA15:AA17"/>
     <mergeCell ref="T22:U22"/>
     <mergeCell ref="AC15:AC17"/>
-    <mergeCell ref="AX20:AX21"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
     <mergeCell ref="AV20:AV21"/>
-    <mergeCell ref="AX22:AX23"/>
     <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AS24:AS25"/>
     <mergeCell ref="AD15:AD17"/>
@@ -3690,7 +3547,6 @@
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="O18:O21"/>
     <mergeCell ref="M18:N21"/>
-    <mergeCell ref="AY22:AY23"/>
     <mergeCell ref="AN18:AN19"/>
     <mergeCell ref="A1:R2"/>
     <mergeCell ref="AL15:AL17"/>
@@ -3701,8 +3557,6 @@
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
     <mergeCell ref="AV24:AV25"/>
-    <mergeCell ref="AX24:AX25"/>
-    <mergeCell ref="AX18:AX19"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
@@ -3711,7 +3565,6 @@
     <mergeCell ref="AV26:AV27"/>
     <mergeCell ref="T19:U19"/>
     <mergeCell ref="AU15:AU17"/>
-    <mergeCell ref="AW15:AW17"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
@@ -3720,19 +3573,16 @@
     <mergeCell ref="P29:Q29"/>
     <mergeCell ref="I15:J17"/>
     <mergeCell ref="C18:D29"/>
-    <mergeCell ref="AY26:AY27"/>
     <mergeCell ref="A15:B17"/>
     <mergeCell ref="K15:L17"/>
     <mergeCell ref="E18:F29"/>
     <mergeCell ref="W23:X27"/>
     <mergeCell ref="T20:U20"/>
-    <mergeCell ref="AM13:AY14"/>
     <mergeCell ref="I18:J21"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="Y27:Y29"/>
     <mergeCell ref="W18:X21"/>
     <mergeCell ref="K6:T6"/>
-    <mergeCell ref="AW18:AW19"/>
     <mergeCell ref="AB13:AL14"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="G10:H10"/>
@@ -3744,8 +3594,6 @@
     <mergeCell ref="Z15:Z17"/>
     <mergeCell ref="AQ18:AQ19"/>
     <mergeCell ref="AB15:AB17"/>
-    <mergeCell ref="AW20:AW21"/>
-    <mergeCell ref="AY20:AY21"/>
     <mergeCell ref="R21:S21"/>
     <mergeCell ref="T21:U21"/>
     <mergeCell ref="A10:C10"/>
@@ -3755,7 +3603,6 @@
     <mergeCell ref="Y15:Y17"/>
     <mergeCell ref="P26:Q27"/>
     <mergeCell ref="T26:U26"/>
-    <mergeCell ref="AW22:AW23"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
@@ -3764,7 +3611,6 @@
     <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>
-    <mergeCell ref="AX26:AX27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>